<commit_message>
test-40: конвейер 2026-08-27 (run 33082752215)
</commit_message>
<xml_diff>
--- a/output/Тест40_2026-08-27.xlsx
+++ b/output/Тест40_2026-08-27.xlsx
@@ -578,15 +578,39 @@
       <c r="G2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>xn--b1aaegg8akarn3job.xn--p1ai</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Прием (осмотр, консультация) врача-косметолога первичный»</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>похож</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>гинеколог, дерматовенеролог, косметолог, онколог, терапевт, хирург</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -632,15 +656,39 @@
       <c r="G3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>stomatolorica.ru</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>стоматолог</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -694,7 +742,7 @@
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
@@ -732,15 +780,39 @@
       <c r="G5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>8-nn.ru</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Документы оформляются на бланках установленного образца. Все филиалы имеют государственную лицензию на осуществление медицинской деятельности» (https://8-nn.ru)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>похож</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматовенеролог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, стоматолог, терапевт, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
@@ -848,15 +920,39 @@
       <c r="G7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>a-clinik.ru</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>гинеколог, дерматолог, косметолог, онкодерматолог, онколог, терапевт, уролог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
@@ -902,7 +998,7 @@
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
@@ -1012,7 +1108,7 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
@@ -1058,7 +1154,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились (гибко)</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
@@ -1104,7 +1200,7 @@
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
@@ -1212,15 +1308,39 @@
       <c r="G14" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>a2med-stomat.ru</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области» (https://a2med-stomat.ru)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>стоматолог, терапевт, хирург</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
@@ -1266,7 +1386,7 @@
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
@@ -1374,15 +1494,39 @@
       <c r="G17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>ava-kazan.ru</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Прием (осмотр, консультация) аллерголога-иммунолога повторный (ДЕТСКИЙ ПРИЕМ)»</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматовенеролог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, ревматолог, терапевт, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились (гибко)</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
@@ -1568,7 +1712,7 @@
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
@@ -1614,7 +1758,7 @@
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -1668,7 +1812,7 @@
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
@@ -1714,7 +1858,7 @@
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
@@ -2110,7 +2254,7 @@
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились (гибко)</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
@@ -2156,7 +2300,7 @@
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
@@ -2202,7 +2346,7 @@
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились (гибко)</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
@@ -2240,15 +2384,23 @@
       <c r="G32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>avtokom54.ru</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr"/>
@@ -2286,15 +2438,39 @@
       <c r="G33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>avtor-e.ru</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>дерматолог, косметолог, психотерапевт, терапевт, трихолог, хирург</t>
+        </is>
+      </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr"/>
@@ -2340,7 +2516,7 @@
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr"/>
@@ -2386,7 +2562,7 @@
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr"/>
@@ -2432,7 +2608,7 @@
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr"/>
@@ -2478,7 +2654,7 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr"/>
@@ -2602,7 +2778,7 @@
       <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились (гибко)</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr"/>
@@ -2640,15 +2816,39 @@
       <c r="G40" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>azbuka-samara.ru</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтеролог, дерматолог, невролог, отоларинголог, офтальмолог, педиатр, стоматолог, терапевт, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr"/>
@@ -2686,15 +2886,39 @@
       <c r="G41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>azbuka-samara.ru</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтеролог, дерматолог, невролог, отоларинголог, офтальмолог, педиатр, стоматолог, терапевт, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr"/>
@@ -5317,7 +5541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5356,24 +5580,288 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>#ЗДОРОВЬЯВСЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0278947517</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>xn--b1aaegg8akarn3job.xn--p1ai</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: xn--b1aaegg8akarn3job.xn--p1ai (страниц скачано: 3)
+TITLE: #ЗдоровьяВсем
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
++7 (919) 603-57-97 | Главная | О нашей клинике | Специалисты центра | Нормативные документы | Вышестоящие организации | Фотогалерея | Услуги и цены | Гинекология | Косметология | Онкология | УЗИ-диагностика | Номенклатура и цены | Акции и скидки | Пациентам | Публикации | Отзывы | Видеоролик о клинике «#ЗдоровьяВсем» | Нигманов Финат Гилевич Директор | Зайнуллин Финар Динарович онколог | Султанова Айгуль Мунировна Медицинская сестра | Нуриева Эльвира Айратовна Косметолог | Вербицкая Елена Борисовна Акушер-гениколог, УЗМ-диагностика | Нигманова Гульнур Хамзеевна Онколог-маммолог | Карачурина Ольга Александровна Медицинская сестра | г. Уфа, ул. Ленина, 156, этаж 1 | zdor.vsem@yandex.ru | Политика обработки персональных данных | Согласие на обработку персональных данных | Политикой обработки персональных данных
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://xn--b1aaegg8akarn3job.xn--p1ai:
+    «г. Уфа, ул. Ленина, 156, этаж 1»
+    «г. Уфа, ул. Ленина, 156, этаж 1»
+  https://xn--b1aaegg8akarn3job.xn--p1ai/uslugi-i-ceny/kosmetologija:
+    «г. Уфа, ул. Ленина, 156, этаж 1»
+    «г. Уфа, ул. Ленина, 156, этаж 1»
+  https://xn--b1aaegg8akarn3job.xn--p1ai/uslugi-i-ceny/onkologija:
+    «г. Уфа, ул. Ленина, 156, этаж 1»
+    «г. Уфа, ул. Ленина, 156, этаж 1»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): гинеколог, дерматовенеролог, косметолог, онколог, терапевт, хирург
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматовенеролог, косметолог, косметология
+ПОЗИЦИИ ПРАЙСА (первые 30 из 37):
+  Цитологическое исследование микропрепарата кожи — 1500
+  Патолого-анатомическое исследование биопсийного (операционного) материала кожи — 1500
+  Биопсия кожи — 1500
+  Подкожное введение лекарственных препаратов — 500
+  Соскоб кожи — 1500
+  Инъекционное введение лекарственных препаратов в очаг поражения кожи — 1000
+  Очищение кожи лица и шеи — 1000
+  Вапоризация кожи лица — 1000
+  Удаление камедонов кожи — 1500
+  Удаление милиумов кожи — 1500
+  Проведение эпиляции — 1000
+  Удаление сосудистой мальформации — 2500
+  Удаление звездчатой ангиомы — 1000
+  Удаление телеангиоэктазий — 1000
+  Удаление контагиозных моллюсков — 1000
+  Удаление татуировки — 500
+  Удаление ногтевых пластинок — 2000
+  Удаление ногтевой пластинки при помощи лазера — 2000
+  Удаление мозоли — 1500
+  Удаление ксантелазм век — 2000
+  Ультразвуковое лечение кожи — 1000
+  Ультразвуковой пилинг — 1500
+  Лазерная шлифовка кожи — 500
+  Лазерная деструкция ткани кожи — 2500
+  Лазерная коагуляция телеангиоэктазий — 2000
+  Прием (осмотр, консультация) врача-косметолога первичный — 1090
+  Пальпация молочных желез — 500
+  Цитологическое исследование отделяемого из соска молочной железы — 1500
+  Биопсия молочной железы чрескожная — 1500
+  Вскрытие панариция — 1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>3Д ДИАГНОСТИКА, ООО</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>5905280410</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>stomatolorica.ru</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: stomatolorica.ru (страниц скачано: 5)
+TITLE: 3D стоматологическая диагностика в Перми - Главная
+DESCRIPTION: Независимые центры трехмерной диагностики
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+Наши центры | О центрах | Сотрудники | Лицензии и сертификаты | Паспорт зубов | Пациентам | Справка в налоговую | Документы | Памятка для родителей на посещение Стоматолорики | Вопрос-Ответ | Отзывы пациентов | Реквизиты | Услуги | Врачу | Направление на рентгенологическое исследование | Отзывы врачей | Технология | Новости и акции | Контакты | Запись онлайн | 8 909-731-03-99 | Назад | info@stomatolorika.ru | Prev | Next | Габитов Альберт Талгатович | Габитов Игорь Талгатович | +7 342 248-02-33 | +7 909-731-03-99 | Компания | Специалисты | Филиалы | Пациенту | Политика конфиденциальности | Бланк направления | Лицензии | Конусно-лучевая компьютерная томография | Все услуги | Все специалисты центра | Подробности | Все филиалы
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  https://stomatolorica.ru: Здоровье для всей семьи | Наши специалисты | О компании | Адреса центров
+  https://stomatolorica.ru/services: Услуги
+  https://stomatolorica.ru/services/konusno-luchevaya-kompyuternaya-tomografiya: Главная
+  https://stomatolorica.ru/services/pasport-zubov: Главная
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://stomatolorica.ru:
+    «г. Пермь, ул. Революции, 21 , тел. 248-02-33»
+    «г. Пермь, Комсомольский проспект, 40, тел. 248-02-33»
+    «г. Пермь, ул. Ленина, 92, тел. 248-02-33»
+    «г. Пермь, ул. Луначарского, 34»
+    «Лицензии и сертификаты»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+    «ул. Революции, 21»
+    «ул. Луначарского, 34»
+    «ул. Луначарского, 34»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+  https://stomatolorica.ru/services:
+    «г. Пермь, ул. Революции, 21 , тел. 248-02-33»
+    «г. Пермь, Комсомольский проспект, 40, тел. 248-02-33»
+    «г. Пермь, ул. Ленина, 92, тел. 248-02-33»
+    «г. Пермь, ул. Луначарского, 34»
+    «Лицензии и сертификаты»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+    «ул. Революции, 21»
+    «ул. Луначарского, 34»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+    «ул. Революции, 21»
+  https://stomatolorica.ru/services/konusno-luchevaya-kompyuternaya-tomografiya:
+    «г. Пермь, ул. Революции, 21 , тел. 248-02-33»
+    «г. Пермь, Комсомольский проспект, 40, тел. 248-02-33»
+    «г. Пермь, ул. Ленина, 92, тел. 248-02-33»
+    «г. Пермь, ул. Луначарского, 34»
+    «Лицензии и сертификаты»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+    «ул. Революции, 21»
+    «ул. Луначарского, 34»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+    «ул. Революции, 21»
+  https://stomatolorica.ru/services/pasport-zubov:
+    «г. Пермь, ул. Революции, 21 , тел. 248-02-33»
+    «г. Пермь, Комсомольский проспект, 40, тел. 248-02-33»
+    «г. Пермь, ул. Ленина, 92, тел. 248-02-33»
+    «г. Пермь, ул. Луначарского, 34»
+    «Лицензии и сертификаты»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+    «ул. Революции, 21»
+    «ул. Луначарского, 34»
+    «ул. Ленина, 92»
+    «ул. Комсомольский проспект, 40»
+    «ул. Революции, 21»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): стоматолог
+ЛИЦЕНЗИЯ (строка с сайта): «Наши центры О центрах Сотрудники Лицензии и сертификаты | Паспорт зубов | Пациентам Справка в налоговую Документы Памятка для родителей на посещение Стоматолорики Вопрос-Ответ Отзывы пациентов Реквизи» (https://stomatolorica.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>8НН, ООО</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>5260143507</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>8-nn.ru</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: 8-nn.ru (страниц скачано: 5)
+TITLE: Медицинский центр в Нижнем Новгороде
+DESCRIPTION: Медицинский центр в Нижнем Новгороде. Медицинский центр «МЕДЭКСПРЕСС» (ООО «8НН») и сеть медицинских клиник «Женский центр» (ООО "Женский центр") уже 20 лет лидируют в области медицины, успешно помогая жителям г. Нижнего Новгорода, Нижегородской области, и других регионов Российской Федерации.
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+center@8-nn.ru | +7 (831) 411-11-11 | Запись на приём | О нас | Информация о медицинских работниках | Контролирующие органы | Диагностика | Маммография | УЗИ | УЗИ органов брюшной полости | УЗИ печени | УЗИ почек | УЗИ сердца | УЗИ поджелудочной железы | УЗИ сосудов и вен | УЗИ щитовидной железы | УЗИ желчного пузыря | УЗИ суставов | УЗИ органов малого таза | УЗИ надпочечников | УЗИ мягких тканей | УЗИ мочевого пузыря | УЗИ молочных желез | УЗИ лимфатических узлов | УЗИ горла и гортани | УЗИ слюнных желез | УЗИ простаты у мужчин | УЗИ селезенки | УЗИ позвоночника | УЗИ головного мозга | ЭКГ-мониторирование | Электрокардиография (ЭКГ) | Рентгенология | CHECK-UP (Комплексное обследование организма) | Функциональная диагностика | Гистеросальпингография | Гистероскопия | Колоноскопия | Кольпоскопия | ФГДС | Эластография | ЭЭГ | Лаборатория | Анализы лабораторные | Анализы на коронавирус | Гематологические исследования | Биохимические исследования | Гормональные исследования | Аллергопанель | Иммунологические исследования | Исследования мочи | Исследования кала | Цитологические исследования | Гистологические исследования | Профильные лабораторные исследования | Онкоскрининг | Инфекционные заболевания | Комплексные исследования | Онкомаркеры и онкологические исследования | Бактериальные инфекции | Паразитарные инфекции | Грибковые инфекции | Справки | Официальные больничные листы | Справка 003-В/у для ГИБДД | Оформить медсправку для приема и устройства на работу | Справки для учебы | Медсправки для детей | Медсправки для занятия спортом | Медсправки для отдыхающих | Справка об отсутствии covid-19 | Другие медсправки | Медкнижки | Гостиничному персоналу | Медицинским работникам | Работникам бань и саун | Работникам образовательных учреждений | Работникам общественного питания | Для организаций | Поликлинический центр | Услуги | Акушерство и гинекология | Медикаментозный аборт | Косметология | Маммология | Стоматология | Процедурный кабинет | Услуги по ОМС | Врачи | Уролог | Акушер‑гинеколог | Медикаментозное прерывание беременности | Маммолог | Рентгенолог | Врач УЗИ | Косметолог | Дерматовенеролог | Эндокринолог | Кардиолог | Невролог | Аллерголог‑иммунолог | Гастроэнтеролог | Офтальмолог | Хирург | Отоларинголог (ЛОР) | Терапевт | Травматолог-ортопед | Флеболог | Инфекционист | Мануальный терапевт | Психиатр | Стоматолог | Имплантология | Терапевтическая стоматология | Ортопедическая стоматология | Хирургическая стоматология | Ортодонтия | Функциональный диагност | Генетик | Диетолог
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  https://8-nn.ru: Медицинский центр «МЕДЭКСПРЕСС» (ООО «8НН»)
+  https://8-nn.ru/oms.html: ОМС | Страховые организации
+  https://8-nn.ru/poliklinicheskij-czentr/uslugi: Услуги
+  https://8-nn.ru/poliklinicheskij-czentr/uslugi/akusherstvo-i-ginekologiya: Акушерство и гинекология | Что находится в компетенции услуг гинеколога | Когда вы должны пройти обследование у гинеколога | Требуется ли особая подготовка перед посещением гинеколога? | На приеме у гинеколога | Чем занимается врач гинеколог | Какие болезни лечит акушер гинеколог | Детали приема у акушера-гинеколога | Когда необходимо обратиться к гинекологу | Вопросы и ответы
+  https://8-nn.ru/poliklinicheskij-czentr/uslugi/akusherstvo-i-ginekologiya/medikamentoznyij-abort.html: Медикаментозный аборт | Медикаментозный аборт: методика и план проведения | Бережная альтернатива хирургическому аборту! | Показания к применению | Побочное действие | Последствия аборта | Постабортный синдром | Вопросы и ответы
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://8-nn.ru:
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Документы оформляются на бланках установленного образца. Все филиалы имеют государственную лицензию на осуществление медицинской деятельности.»
+    «Лицензии»
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Медцентр «МЕДЭКСПРЕСС-8НН» (ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ «8НН», ИНН 5260143507)»
+  https://8-nn.ru/oms.html:
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «603000, г. Нижний Новгород, ул. Белинского, дом 32»
+    «603000, г. Нижний Новгород, ул. Славянская, дом 8»
+    «3. Филиал ООО "Страховая компания "Ингосстрах-М" в г. Н.Новгороде»
+    «603000, г. Нижний Новгород, ул. Новая, дом 34Б»
+    «Лицензии»
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Медцентр «МЕДЭКСПРЕСС-8НН» (ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ «8НН», ИНН 5260143507)»
+  https://8-nn.ru/poliklinicheskij-czentr/uslugi:
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Лицензии»
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Медцентр «МЕДЭКСПРЕСС-8НН» (ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ «8НН», ИНН 5260143507)»
+  https://8-nn.ru/poliklinicheskij-czentr/uslugi/akusherstvo-i-ginekologiya:
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Эндокринные – патологии связанные с гормональными нарушениями в организме женщины»
+    «Нарушения менструального цикла – отсутствие менструации, нерегулярный цикл, слишком обильные или скудные выделения, продолжительный или короткий период, болезненность – все эти признаки могут говорить о развитии патологий эндокринного,»
+    «Лицензии»
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Медцентр «МЕДЭКСПРЕСС-8НН» (ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ «8НН», ИНН 5260143507)»
+  https://8-nn.ru/poliklinicheskij-czentr/uslugi/akusherstvo-i-ginekologiya/medikamentoznyij-abort.html:
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Лицензии»
+    «Нижний Новгород, ул.Германа Лопатина, д.8»
+    «Медцентр «МЕДЭКСПРЕСС-8НН» (ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ «8НН», ИНН 5260143507)»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): аллерголог, гастроэнтеролог, гинеколог, дерматовенеролог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, стоматолог, терапевт, уролог, флеболог, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматовенеролог, косметолог, косметология
+ЛИЦЕНЗИЯ (строка с сайта): «Документы оформляются на бланках установленного образца. Все филиалы имеют государственную лицензию на осуществление медицинской деятельности» (https://8-nn.ru)
+ПОЗИЦИИ ПРАЙСА (первые 30 из 91):
+  Прививка от кори — 500 руб
+  СДЕЛАЙ ТЕСТ - ПРОВЕРЬ ПРИВИТ ИЛИ НЕТ! Тест на наличие антител к вирусу кори lgG — 500 руб
+  Скидка 50% до 31.08.2025 — 2500 руб
+  Остроконечные кондиломы: d до 0,5 см — 50,00 руб
+  Остроконечные кондиломы: d более 0,5 см — 400,00 руб
+  Остроконечные кондиломы: удаление более 30 единиц — 400,00 руб
+  Анестезия ( местное обезболивание) — 300,00 руб
+  Лазердеструкция (обширная) — 5000,00 руб
+  Диагностическая пункционная биопсия — 550,00 руб
+  Санация (обработка) влагалища — 150,00 руб
+  Биопсия шейки матки конхотомом — 350,00 руб
+  Обработка шейки матки — 150,00 руб
+  Введение ВМК — 1000,00 руб
+  Введение ВМК - (Мирена) Без стоимости ВМК — 1500,00 руб
+  Удаление ВМК (простое) — 500,00 руб
+  Биопсия шейки матки ножевая — 1500,00 руб
+  ВМК Миренас контролем УЗИ и обезболиванием — 14500,00 руб
+  Прием доктора медицинских наук — 1200,00 руб
+  Папиллома вульвы последующие — 100,00 руб
+  Консультация гинекологическая при стрессовом недержаниимочи — 300,00 руб
+  Пайпель биопсия шейки матки конхотомом — 1000,00 руб
+  Лазерная деструкция шейки матки d 2 см — 3500,00 руб
+  Хронический эктоцервикоз — 3000,00 руб
+  Эрозированный эктропион — 3000,00 руб
+  Эрозированный эктропион, сложный — 3500,00 руб
+  Лейкоплакия — 2000,00 руб
+  Папиллома шейки матки, последующие единицы — 100,00 руб
+  Пайпель биопсия шейки матки — 1000,00 руб
+  Лейкоплакия сложная — 2500,00 руб
+  Подготовкашейки матки медикаментозная — 2000,00 руб</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>9 МЕСЯЦЕВ, ООО КЛИНИКА</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>1660147957</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>c9m.ru</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>САЙТ: c9m.ru (страниц скачано: 5)
 TITLE: Клиника «9 месяцев» - клиника женского и детского здоровья в Казани
@@ -5483,26 +5971,70 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>А-КЛИНИК, ООО</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>7203547497</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>a-clinik.ru</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: a-clinik.ru (страниц скачано: 1)
+TITLE: A-Клиника| Медицинская клиника
+DESCRIPTION: Дневной стационар, терапия, дерматология, дерматоонкология, амбулаторная хирургия
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+Главная | Врачи | Направления | Восполнение дефицитов | Чекапы | Онкодерматология, хирургия кожи | Маммология | Проктология | Дерматология и косметология | Анализы | Гинекология | Цены | Контакты | Миссия | О клинике | Онлайн запись | Записаться на капельницу | Записаться на чекап | Записаться к врачам | персональных данных | договором оферты | Записаться на приём | Приём терапевта ежедневно | Решаем проблемы с хронической усталостью | УЗИ чекап - 40% | Ежедневный приём онколога | Лечение анемии | Онлайн запись на приём | Онкодерматология и хирургия кожи | Диагностика и лечение заболеваний молочных желез. | Терапия | Первичный приём и комплексная оценка состояния здоровья. | УЗИ | Урология | Эндокринология | Подробнее о врачах | политикой конфиденциальности | КАРТА САЙТА → | ВЕРСИЯ ДЛЯ СЛАБОВИДЯЩИХ → | Политика конфиденциальности | Публичная оферта | Шаблон договора
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://a-clinik.ru:
+    «Номер лицензии:»
+    «ИНН 7203199480»
+    «ОГРН 1077203043060»
+    «г. Тюмень, ул. Циолковского 20а»
+    «Номер лицензии:»
+    «ИНН 7203547497»
+    «ОГРН 1227200019892»
+    «г. Тюмень, ул. Малыгина 4/1»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): гинеколог, дерматолог, косметолог, онкодерматолог, онколог, терапевт, уролог, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, дерматология, дерматоскопия, косметолог, косметология, онкодерматолог, онкодерматология, удаление новообразований
+ЛИЦЕНЗИЯ (строка с сайта): «Номер лицензии» (https://a-clinik.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>А-МЦ УЛЬТРАМЕД, ООО</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>5256051451</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>ultramed-nn.ru</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>САЙТ: ultramed-nn.ru (страниц скачано: 5)
 TITLE: Сеть клиник «Ультрамед» в Нижнем Новгороде
@@ -5617,26 +6149,26 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+    <row r="8">
+      <c r="A8" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>А2МЕД ЧЕЛЯБИНСК, ООО</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>7451374192</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>parkmed.ru</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>САЙТ: parkmed.ru (страниц скачано: 4)
 TITLE: Клиника Парк-Мед | МРТ в Челябинске. Цены от 2000 рублей
@@ -5670,26 +6202,89 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>А2МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>6317157682</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>a2med-stomat.ru</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: a2med-stomat.ru (страниц скачано: 5)
+TITLE: Стоматология A2MED в Самаре — лечение зубов и имплантация
+DESCRIPTION: A2MED — современная стоматология в Самаре. Безболезненное лечение, имплантация, чистка и выравнивание зубов. Индивидуальный подход и точная диагностика.
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+СТОМАТОЛОГИЧЕСКАЯ КЛИНИКА | Услуги | Специалисты | Отзывы | Контакты | Акции | Наши работы | +7 (987) 980 00 30 | +7 (846) 313 03 03 | Записаться | Запишись сейчас | Выбрать услугу | Выбрать дату | Записаться со скидкой | политикой конфиденциальности | обработку персональных данных | Телефон отделения +7 (987) 980 00 30 | Единый номер A2Мед +7 (846) 313 03 03 | Дачная ул., 24, этаж 6 | Политика конфидициальности и обработки персональных данных | mirniydev
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  https://a2med-stomat.ru: Стоматология | Лечение без стресса | Полезные видео | Ознакомьтесь с услугами стоматологии А2MED | Команда замечательных специалистов | Наши работы | Отзывы пациентов | Ознакомьтесь с актуальными АКЦИЯМИ | Сертификаты и награды специалистов | Оставьте заявку — мы свяжемся с вами | Контакты
+  https://a2med-stomat.ru/?service=cmr7yhlbt000001pavmih441l: Стоматология | Лечение без стресса | Полезные видео | Ознакомьтесь с услугами стоматологии А2MED | Команда замечательных специалистов | Наши работы | Отзывы пациентов | Ознакомьтесь с актуальными АКЦИЯМИ | Сертификаты и награды специалистов | Оставьте заявку — мы свяжемся с вами | Контакты
+  https://a2med-stomat.ru/?service=cmr7yjlyl000101pa5qaq8xnq: Стоматология | Лечение без стресса | Полезные видео | Ознакомьтесь с услугами стоматологии А2MED | Команда замечательных специалистов | Наши работы | Отзывы пациентов | Ознакомьтесь с актуальными АКЦИЯМИ | Сертификаты и награды специалистов | Оставьте заявку — мы свяжемся с вами | Контакты
+  https://a2med-stomat.ru/?service=cmr7yl89a000201pamrq14mki: Стоматология | Лечение без стресса | Полезные видео | Ознакомьтесь с услугами стоматологии А2MED | Команда замечательных специалистов | Наши работы | Отзывы пациентов | Ознакомьтесь с актуальными АКЦИЯМИ | Сертификаты и награды специалистов | Оставьте заявку — мы свяжемся с вами | Контакты
+  https://a2med-stomat.ru/?service=cmr7ymlvd000301paex1wnkgk: Стоматология | Лечение без стресса | Полезные видео | Ознакомьтесь с услугами стоматологии А2MED | Команда замечательных специалистов | Наши работы | Отзывы пациентов | Ознакомьтесь с актуальными АКЦИЯМИ | Сертификаты и награды специалистов | Оставьте заявку — мы свяжемся с вами | Контакты
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://a2med-stomat.ru:
+    «Дачная ул., 24, этаж 6»
+    «Дачная ул., 24, этаж 6»
+    «ООО "А2Мед Самара" ИНН 6315023806 ОГРН 1186313048052»
+    «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области.»
+  https://a2med-stomat.ru/?service=cmr7yhlbt000001pavmih441l:
+    «Дачная ул., 24, этаж 6»
+    «Дачная ул., 24, этаж 6»
+    «ООО "А2Мед Самара" ИНН 6315023806 ОГРН 1186313048052»
+    «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области.»
+  https://a2med-stomat.ru/?service=cmr7yjlyl000101pa5qaq8xnq:
+    «Дачная ул., 24, этаж 6»
+    «Дачная ул., 24, этаж 6»
+    «ООО "А2Мед Самара" ИНН 6315023806 ОГРН 1186313048052»
+    «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области.»
+  https://a2med-stomat.ru/?service=cmr7yl89a000201pamrq14mki:
+    «Дачная ул., 24, этаж 6»
+    «Дачная ул., 24, этаж 6»
+    «ООО "А2Мед Самара" ИНН 6315023806 ОГРН 1186313048052»
+    «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области.»
+  https://a2med-stomat.ru/?service=cmr7ymlvd000301paex1wnkgk:
+    «Дачная ул., 24, этаж 6»
+    «Дачная ул., 24, этаж 6»
+    «ООО "А2Мед Самара" ИНН 6315023806 ОГРН 1186313048052»
+    «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области.»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): стоматолог, терапевт, хирург
+ЛИЦЕНЗИЯ (строка с сайта): «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области» (https://a2med-stomat.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>6165200482</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>аве-вита.рф</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>САЙТ: аве-вита.рф (страниц скачано: 3)
 TITLE: Поликлиника «АвеВита» в Ростове-на-Дону
@@ -5734,26 +6329,136 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>АВА-КАЗАНЬ, АО</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>1655146267</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ava-kazan.ru</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: ava-kazan.ru (страниц скачано: 5)
+TITLE: Клиника внимательной медицины "Скандинавия"
+DESCRIPTION: Клиника внимательной медицины "Скандинавия". Записаться на консультацию по номеру 8 (843) 200-10-65 круглосуточно.
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+ЭКО Скандинавия АВА-ПЕТЕР | Услуги | Поликлиника | Педиатрия | Диагностика | Гинекология | Оперативная гинекология | Ведение беременности | Гематология | Кардиология | Неврология | Онкология, маммология | Офтальмология | Флебология | Терапия | Травматология и ортопедия | Урология | Хирургия | Эндокринология | Стационар | Чек-апы | Детские чек-апы | Акции | Врачи | Цены | Роддом | Грудное вскармливание | Криоконсервация стволовых клеток из пуповинной крови | Мягкие роды | Партнерские роды | Реанимация новорожденных | Роды по стандартам Халяль | Уход за новорожденными | Фотосессия новорожденных малышей | Что входит в договор на роды? | Экскурсия в роддом | Эпидуральная анестезия при родах | Пластическая хирургия | Пластика груди | Пластика лица | Пластика тела | Лечение ожирения | Пластика после родов | Коррекция рубцов и шрамов | Липосакция и липофилинг | Медицинский туризм | Косметология | Аппаратная/уходовая косметология | Дефекты кожи | Инъекции | Контурная пластика | ЭКО | Подготовка к ЭКО | Беспроцентная рассрочка | ЭКО по квотам ОМС | ЭКО по ОМС для жителей других регионов РФ | Гистероскопия одного дня | Какие анализы и документы нужны для ЭКО | О компании | О клинике | Контакты | Руководство | Специалисты | Виртуальный тур | Лицензии | Органы надзора | Нормативно-правовые документы | Отчеты | Отзывы | Пациентам | Пресса о нас | Корпоративным клиентам | Оформление в клинике | Отели-партнеры | Подготовка к анастезии и операциям | Подготовка к диагностическим исследованиям и манипуляциям | Правила сдачи анализов | Подготовка к лабораторным исследованиям | Оформление налогового вычета | Режим приема билогического материала | +7 (843) 200-10-65 | info@avakazan.ru | 8 (843) 200-10-65 | обратный звонок | Записаться | Запись | Беременность и роды | Эстетическая медицина | Поиск по сайту... | Беременность | Вакцинация | МРТ | Лабораторные исследования | Лечение бесплодия | Оформление | Налоговый вычет | Подготовка к исследованиям | Подготовка к анестезии | Подготовка к манипуляциям | АВА-Петер | Скандинавия Казань | Смотреть | Скачать | Записаться онлайн | Взрослые врачи Прием от 1200 руб | Гинеколог | Терапевт | Онколог | Флеболог | и еще 16 специалистов... | Детские врачи Прием от 1200 руб | Педиатр | Детский невролог | Массаж | Аллерголог-иммунолог | и еще 13 специалистов... | УЗИ | Рентген | Чек-ап | и еще 3 услуги...
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  https://ava-kazan.ru: Клиника Скандинавия Казань | Услуги клиники «Скандинавия» (АВА-Казань) | Познакомьтесь с нашей клиникой | Наши основные качества | Отправить заявку
+  https://ava-kazan.ru/price: Стоимость услуг | Отправить заявку
+  https://ava-kazan.ru/structure: Направления | Отправить заявку
+  https://ava-kazan.ru/structure/diagnostika/uslugi-uzi: Ультразвуковые исследования (УЗИ) | Акции | О направлении | Виды УЗИ | Когда назначают УЗИ | Врачи | Отправить заявку
+  https://ava-kazan.ru/clinic/specialist: Специалисты | Отправить заявку
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://ava-kazan.ru:
+    «Криоконсервация стволовых клеток из пуповинной крови»
+    «Лицензии»
+    «Лицензии»
+    «г. Казань, ул. Профсоюзная/Астрономическая, д. 19/15»
+    «Режим работы»
+    «Лицензии»
+    «Лицензия»
+    «Зиннуров Фидель Равильевич»
+    «Пономарева Инна Витальевна»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+  https://ava-kazan.ru/price:
+    «Криоконсервация стволовых клеток из пуповинной крови»
+    «Лицензии»
+    «Лицензии»
+    «Лицензии»
+    «Лицензия»
+    «Зиннуров Фидель Равильевич»
+    «Пономарева Инна Витальевна»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+  https://ava-kazan.ru/structure:
+    «Криоконсервация стволовых клеток из пуповинной крови»
+    «Лицензии»
+    «Лицензии»
+    «Лицензии»
+    «Лицензия»
+    «Зиннуров Фидель Равильевич»
+    «Пономарева Инна Витальевна»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+  https://ava-kazan.ru/structure/diagnostika/uslugi-uzi:
+    «Криоконсервация стволовых клеток из пуповинной крови»
+    «Лицензии»
+    «Лицензии»
+    «Лицензии»
+    «Лицензия»
+    «Зиннуров Фидель Равильевич»
+    «Пономарева Инна Витальевна»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+  https://ava-kazan.ru/clinic/specialist:
+    «Криоконсервация стволовых клеток из пуповинной крови»
+    «Лицензии»
+    «Лицензии»
+    «Лицензии»
+    «Лицензия»
+    «Зиннуров Фидель Равильевич»
+    «Пономарева Инна Витальевна»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+    «В соответствии с Федеральным законом от 27.07.2006 г. № 152-ФЗ «О персональных данных»,»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): аллерголог, гастроэнтеролог, гинеколог, дерматовенеролог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, ревматолог, терапевт, уролог, флеболог, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматовенеролог, дерматолог, дерматология, косметолог, косметология
+ЛИЦЕНЗИЯ (строка с сайта): «Лицензии» (https://ava-kazan.ru)
+ПОЗИЦИИ ПРАЙСА (первые 9 из 9):
+  Контурная пластика
+  Прием от — 1200 руб
+  Специализированный прием по плану лечения эндометриоза — 1 300 руб
+  Профилактический прием (осмотр, консультация) акушера-гинеколога — 1 700 руб
+  Повторный прием по медикаментозному прерыванию беременности — 2 000 руб
+  Прием (осмотр, консультация) аллерголога-иммунолога повторный (ДЕТСКИЙ ПРИЕМ) — 2 400 руб
+  Прием (осмотр, консультация) анестезиолога первичный — 2 900 руб
+  Консультативный прием заведующим отделением Анестезиология-Реанимация — 3 300 руб
+  Поддержание медикаментозной седации (каждые 30 минут) — 2 100 руб</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>5406302509</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>avanta-med.ru</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avanta-med.ru (страниц скачано: 5)
 TITLE: Медицинский центр Аванта-Мед в Новосибирске
@@ -5809,26 +6514,26 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+    <row r="13">
+      <c r="A13" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>АВАНТИС, ООО</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>5402038349</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>avantis-stom.ru</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avantis-stom.ru (страниц скачано: 1)
 TITLE: Брекеты в Новосибирске: цена на установку от 14900 рублей
@@ -5856,26 +6561,26 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>6658006884</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>aviodent.ru</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>САЙТ: aviodent.ru (страниц скачано: 2)
 TITLE: Сеть стоматологических клиник Доктора Мансурского | Платная стоматология в в Екатеринбурге
@@ -5907,26 +6612,26 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>5406513676</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>avismed-nsk.ru</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avismed-nsk.ru (страниц скачано: 5)
 TITLE: Лечебно-диагностический центр «АвисМед»
@@ -5973,26 +6678,26 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+    <row r="16">
+      <c r="A16" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>1653000230</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>avicenna-endocrin.ru</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna-endocrin.ru (страниц скачано: 5)
 TITLE: Клиника профессора Анчиковой - Главная
@@ -6052,26 +6757,26 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>5406137478</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>avicenna-nsk.ru</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna-nsk.ru (страниц скачано: 4)
 TITLE: Медицинский центр "АВИЦЕННА" - частная клиника мирового уровня в Новосибирске
@@ -6103,26 +6808,26 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>7204082420</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>avicenna72.ru</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna72.ru (страниц скачано: 5)
 TITLE: Многопрофильный медицинский центр в Тюмени — «Авиценна»
@@ -6229,26 +6934,119 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>5407494063</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>avtor-e.ru</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: avtor-e.ru (страниц скачано: 5)
+TITLE: Клиника врачебной косметологии в Новосибирске | Услуги пластической хирургии в авторской клинике доктора Егорова
+DESCRIPTION: Клиника пластической хирургии и врачебной косметологии в Новосибирске узнать цены можно по телефону ☎ +7 (383) 209-06-89.
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
++7 383 209 06 89 | +7 800 511 81 89 | АВТОРСКАЯ КЛИНИКА ДОКТОРА ЕГОРОВА | КЛИНИКА ПЛАСТИЧЕСКОЙ ХИРУРГИИ И ВРАЧЕБНОЙ КОСМЕТОЛОГИИ | ЗАПИСАТЬСЯ НА ПРИЁМ | согласием на обработку персональных данных | Пластическая хирургия | Пластика груди | ▪️Реконструктивная маммопластика | ▪️Подтяжка груди | ▪️Уменьшение груди | ▪️Имплантация облегченными имплантатами B-Lite | Пластика тела | ▪️Липосакция | ▪️Абдоминопластика | Пластика лица | ▪️Подтяжка лица | ▪️Блефаропластика | Косметология | Инъекционная | Аппаратная | Увеличение губ | Контурная пластика лица | Услуги клиники | Диетолог | Сомнолог | Биоимпедансометрия | Похудение с препаратом Тирзетта | Цены | Прайс на пластические операции | Прайс на услуги косметолога | Прайс на прочие услуги клиники | О клинике | Наши врачи | Подготовка к операции | Правовая информация | СМИ | Вопросы и ответы | Отзывы | Контакты | Фотогалерея | До \ После | Фотоотзывы пациентов | Рабочий процесс | ▫️Реконструктивная маммопластика | ▫️Подтяжка груди | ▫️Уменьшение груди | ▫️Имплантация облегченными имплантатами B-Lite | ▫️Липосакция | ▫️Абдоминопластика | ▫️Подтяжка лица | ▫️Блефаропластика | Прием врача-диетолога | Прием врача-сомнолога | Запись на приём | Диетология | Сомнология | Абдоминопластика | Подробнее → | Липосакция | Лифтинг лица | Блефаропластика | Подтяжка груди | Увеличение груди | Егоров Вадим Анатольевич | Кереленская Наталья Валерьевна | Иванова Яна Анатольевна | Лицензия №1 | Адреса осуществления деятельности | Приложение к лицензии №1 | Приложение к лицензии №2-1 | Приложение к лицензии №2-2 | Приложение к лицензии №2-3 | Лицензия №2 | политикой обработки персональных данных | Отзывы о нас на Флампе | +7 (383) 209-06-89 | 8 (800) 511-81-89 | info@avtor-e.ru | Согласие на обработку персональных данных
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  https://avtor-e.ru: Клиника врачебной косметологии и пластической хирургии | Кратко о наших услугах | Мы специализируемся: | Наши специалисты | Отзывы | Фотографии счастливых пациенток
+  https://avtor-e.ru/ceni-na-kosmetologicheskie-uslugi: Цены на косметологические услуги
+  https://avtor-e.ru/ceni-na-prochie-uslugi: Цены на услуги сомнолога и диетолога в Новосибирске
+  https://avtor-e.ru/price-plastika: Цены на пластические операции
+  https://avtor-e.ru/vrachi: Врачи | Наши преимущества: | Отзывы
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://avtor-e.ru:
+    «Body-Jet - инновационный способ липосакции, который позволяет избавиться от лишних жировых клеток, не нанося вред организму.»
+    «Лицензии»
+    «Лицензия №1»
+    «Приложение к лицензии №1»
+    «Приложение к лицензии №2-1»
+    «Приложение к лицензии №2-2»
+    «Приложение к лицензии №2-3»
+    «Лицензия №2»
+    «г. Новосибирск ,»
+    «ул. 1905 года, д. 85/2»
+  https://avtor-e.ru/ceni-na-kosmetologicheskie-uslugi:
+    «г. Новосибирск ,»
+    «ул. 1905 года, д. 85/2»
+  https://avtor-e.ru/ceni-na-prochie-uslugi:
+    «г. Новосибирск ,»
+    «ул. 1905 года, д. 85/2»
+  https://avtor-e.ru/price-plastika:
+    «г. Новосибирск ,»
+    «ул. 1905 года, д. 85/2»
+  https://avtor-e.ru/vrachi:
+    «г. Новосибирск ,»
+    «ул. 1905 года, д. 85/2»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): дерматолог, косметолог, психотерапевт, терапевт, трихолог, хирург
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, косметолог, косметология, трихолог, удаление новообразований
+ЛИЦЕНЗИЯ (строка с сайта): «Лицензии» (https://avtor-e.ru)
+ПОЗИЦИИ ПРАЙСА (первые 30 из 101):
+  БИОРЕВИТАЛИЗАЦИЯ
+  GENYAL GENIALLIFT (1.0 мл) — 12 100 руб
+  ELDERMAFIL COLLAGEN+ACTIVATOR (5.0мл) — 22 000 руб
+  Диспорт 1 Ед — 150 руб
+  Ксеомин 1 Ед — 370 руб
+  КОНТУРНАЯ ПЛАСТИКА
+  TEOSYAL PureSense Redensity II (1,0 мл) — 28 900 руб
+  GENYAL VOLUMAE (1,0 мл.) — 18 400 руб
+  FIBROLIFT SOFT (10,0 мл.) — 23 600 руб
+  XSPURT Finale - 1,1мл — 13 200 руб
+  RADIESSE - гель на основе гидроксиапатита кальция, предназначенный для долговременной коррекции морщин (шприц 1,5 мл) — 29 400 руб
+  ELDERMAFILL 3G-In Volume - 5 мл — 11 600 руб
+  МЕЗОТЕРАПИЯ ЛИЦА
+  ELDERMAFILL Lipo-body ampoule (5,0 мл) — 2 100 руб.
+  ELDERMAFILL HTL-T ampoule - Липомоделирующий лосьон для контуров лица и тела (5,0 мл.) — 2 100 руб.
+  ELDERMAFILL V-up gravitation ampoule - Аnti-age лосьон с полинуклеотидами для обновления структуры кожи лица и тела. Ока — 2 100 руб.
+  HAIR X — Мезораствор для волос (4,0 мл.) — 1 600 руб.
+  ELDERMAFILL Volume Ampoule (5,0 мл) — 1 800 руб.
+  3D-мезонити (2,5 см.) - 1 процедура — 11 000 руб
+  3D-мезонити скрученные (5 см.) - 1 процедура — 14 500 руб
+  8D-мезонити Dr.COG - 1 процедура — 15 300 руб
+  ПИЛИНГИ
+  Манделак (DERMATIME-Mandelic A40 Peeling Solution-Раствор для пилинга), 10 мл — 3 800 руб
+  Пилинг Джесснера (DERMATIME - JM1 Peeling Solution-Раствор-пилинг), 10 мл — 3 800 руб
+  Biomatrix GLYCOLIN-50 Пилинг для лица с гликолевой кислотой, 10 мл — 3 800 руб
+  Массаж лица — 3 500 руб
+  Комбинированная чистка лица — 4 000 руб
+  Микротоковая терапия на аппарате Skin Master — 2500 руб
+  Лицо, не включая область век и шеи — 12 600 руб
+  Верхняя часть лица (лоб, глаза, височная область) — 10 500 руб</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>АГК, ООО</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>2461016768</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>agk24.ru</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>САЙТ: agk24.ru (страниц скачано: 5)
 TITLE: Вопросы женского и мужского здоровья | ООО "Андро-гинекологическая клиника", г. Красноярск
@@ -6294,6 +7092,110 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>azbuka-samara.ru</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: azbuka-samara.ru (страниц скачано: 3)
+TITLE: Семейный медицинский центр Самара 🏥 | Детский развивающий клуб
+DESCRIPTION: Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+О нас | Документы | Услуги | Наши врачи | Акции | Отзывы | Контакты | 8 (846) 231-27-04 | 8 (937) 992-27-04 | Детский клуб | Тхэквондо | Проведение детских праздников / аренда зала | Группа подготовки детей к школе от 5 до 7 лет | Семейный медицинский центр | Гастроэнтеролог | Терапевт | УЗИ для детей и взрослых (Эхо КГ) | Психиатр детский | Мануальный терапевт | Эндокринолог | Педиатр | Офтальмолог | Экг | Мед справки | Процедурный кабинет | Отоларинголог | Дерматолог | Невролог | Стоматология для детей и взрослых | Лечение под микроскопом | Компьютерная томография КТ зубов | Удаление зубов и хирургия | Имплантация | Гнатолог (Лечение заболеваний суставов челюсти) | Ортопед (протезирование зубов: коронки, мосты, протезы) | Ортодонт (выравнивание зубов: пластинки, брекеты, капы) | Подробнее... | Узнать больше | 8 (846)330-28-03 | 8 (846)231-27-04 | 8 (937)992-27-04 | a-zdorovya@mail.ru | Политика конфиденциальности | Согласие на обработку ПДн
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr: Семейный медицинский центр | Преимущества семейного медицинского центра
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr/dermatovenerolog: Дерматолог | НАПРАВЛЕНИЯ ЛЕЧЕНИЯ | ЦЕНЫ НА УСЛУГИ
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://azbuka-samara.ru:
+    «Самара, Долотный переулок д. 11»
+    «Самара, Долотный переулок, 11.»
+    «Режим работы»
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr:
+    «Самара, Долотный переулок д. 11»
+    «Самара, Долотный переулок, 11.»
+    «Режим работы»
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr/dermatovenerolog:
+    «Самара, Долотный переулок д. 11»
+    «Самара, Долотный переулок, 11.»
+    «Режим работы»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): гастроэнтеролог, дерматолог, невролог, отоларинголог, офтальмолог, педиатр, стоматолог, терапевт, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, дерматология
+ПОЗИЦИИ ПРАЙСА (первые 4 из 4):
+  Лечение зубов под микроскопом с выгодой до — 6 000 руб
+  Консультация — 2 500
+  Удаление сухой мозоли — 500
+  Анестезия — 200</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>6314040975</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>azbuka-samara.ru</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: azbuka-samara.ru (страниц скачано: 3)
+TITLE: Семейный медицинский центр Самара 🏥 | Детский развивающий клуб
+DESCRIPTION: Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+О нас | Документы | Услуги | Наши врачи | Акции | Отзывы | Контакты | 8 (846) 231-27-04 | 8 (937) 992-27-04 | Детский клуб | Тхэквондо | Проведение детских праздников / аренда зала | Группа подготовки детей к школе от 5 до 7 лет | Семейный медицинский центр | Гастроэнтеролог | Терапевт | УЗИ для детей и взрослых (Эхо КГ) | Психиатр детский | Мануальный терапевт | Эндокринолог | Педиатр | Офтальмолог | Экг | Мед справки | Процедурный кабинет | Отоларинголог | Дерматолог | Невролог | Стоматология для детей и взрослых | Лечение под микроскопом | Компьютерная томография КТ зубов | Удаление зубов и хирургия | Имплантация | Гнатолог (Лечение заболеваний суставов челюсти) | Ортопед (протезирование зубов: коронки, мосты, протезы) | Ортодонт (выравнивание зубов: пластинки, брекеты, капы) | Подробнее... | Узнать больше | 8 (846)330-28-03 | 8 (846)231-27-04 | 8 (937)992-27-04 | a-zdorovya@mail.ru | Политика конфиденциальности | Согласие на обработку ПДн
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr: Семейный медицинский центр | Преимущества семейного медицинского центра
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr/dermatovenerolog: Дерматолог | НАПРАВЛЕНИЯ ЛЕЧЕНИЯ | ЦЕНЫ НА УСЛУГИ
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://azbuka-samara.ru:
+    «Самара, Долотный переулок д. 11»
+    «Самара, Долотный переулок, 11.»
+    «Режим работы»
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr:
+    «Самара, Долотный переулок д. 11»
+    «Самара, Долотный переулок, 11.»
+    «Режим работы»
+  https://azbuka-samara.ru/uslugi/semejnyj-meditsinskij-tsentr/dermatovenerolog:
+    «Самара, Долотный переулок д. 11»
+    «Самара, Долотный переулок, 11.»
+    «Режим работы»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): гастроэнтеролог, дерматолог, невролог, отоларинголог, офтальмолог, педиатр, стоматолог, терапевт, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, дерматология
+ПОЗИЦИИ ПРАЙСА (первые 4 из 4):
+  Лечение зубов под микроскопом с выгодой до — 6 000 руб
+  Консультация — 2 500
+  Удаление сухой мозоли — 500
+  Анестезия — 200</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6305,7 +7207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6362,16 +7264,16 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>9 МЕСЯЦЕВ, ООО КЛИНИКА</t>
+          <t>#ЗДОРОВЬЯВСЕМ, ООО</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1660147957</t>
+          <t>0278947517</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -6391,32 +7293,32 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>гинекология, педиатрия, УЗИ, анализы</t>
+          <t>дерматология, косметология, онкология</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Регистрационный номер лицензии Л041-01181-16/00348727 от 20.04.2020г выдана Министерством здравоохранения РТ</t>
+          <t>Приём врача (специалисты центра), медицинские услуги в прайсе (Цитологическое исследование микропрепарата кожи, Биопсия кожи, Удаление камедонов кожи и т.д.)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>А-МЦ УЛЬТРАМЕД, ООО</t>
+          <t>#ЗДОРОВЬЯВСЕМ, ООО</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>5256051451</t>
+          <t>0278947517</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -6426,32 +7328,32 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>управляющая компания сети клиник</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>акушерство и гинекология, гастроэнтерология, дерматология, кардиология, неврология, онкология, оториноларингология, пульмонология, ревматология, терапия, урология, эндокринология</t>
+          <t>гинекология, косметология, онкология, УЗИ-диагностика</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Прием врача-гинеколога, Прием врача-гастроэнтеролога, Прием врача-дерматолога / дерматовенеролога, Прием врача-кардиолога, Прием врача-невролога, Прием врача-онколога, Лечение ЛОР-заболеваний, Пульмонология, Прием врача-ревматолога, Прием врача-терапевта, Прием врача-уролога, Прием врача-эндокриноло</t>
+          <t>На сайте представлены медицинские услуги, включая косметологию, онкологию и гинекологию. Указан адрес и контактные данные, что подтверждает медицинскую направленность.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>А2МЕД ЧЕЛЯБИНСК, ООО</t>
+          <t>3Д ДИАГНОСТИКА, ООО</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>7451374192</t>
+          <t>5905280410</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -6471,32 +7373,32 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, терапия, урология, эндокринология</t>
+          <t>стоматология</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Миссия клиники Парк Мед заключается в восстановлении и сохранении здоровья, используя современный медицинские технологии, профессионализм, заботу и доверие.</t>
+          <t>Здоровье для всей семьи | Наши специалисты | О компании | Адреса центров</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>АВ ДГТУ, ООО</t>
+          <t>3Д ДИАГНОСТИКА, ООО</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>6165200482</t>
+          <t>5905280410</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -6511,32 +7413,32 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>дерматология, венерология</t>
+          <t>стоматология</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Дерматовенеролог, дерматовенерология в профиле врачей и направлениях</t>
+          <t>Независимые центры трехмерной диагностики. Стоматолог.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>АВАНТА-МЕД, ООО</t>
+          <t>8НН, ООО</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>5406302509</t>
+          <t>5260143507</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -6551,27 +7453,27 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, дерматология, отоларингология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, косметология, стоматология</t>
+          <t>акушерство и гинекология, косметология, маммология, стоматология, общая практика</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+          <t>Документы оформляются на бланках установленного образца. Все филиалы имеют государственную лицензию на осуществление медицинской деятельности.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>АВАНТИС, ООО</t>
+          <t>9 МЕСЯЦЕВ, ООО КЛИНИКА</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>5402038349</t>
+          <t>1660147957</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6586,37 +7488,37 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>ортодонтия</t>
+          <t>гинекология, педиатрия, УЗИ, анализы</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
+          <t>Регистрационный номер лицензии Л041-01181-16/00348727 от 20.04.2020г выдана Министерством здравоохранения РТ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+          <t>9 МЕСЯЦЕВ, ООО КЛИНИКА</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>6658006884</t>
+          <t>1660147957</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -6626,32 +7528,32 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>стоматология</t>
+          <t>гинекология, педиатрия, ведение беременности, терапия, кардиология, эндокринология, снижение веса, офтальмология, вакцинация, урология</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
+          <t>Частная клиника «9 месяцев» в Казани: мед. услуги для взрослых и детей. Консультации, УЗИ, анализы, гинекология, ведение беременности, педиатрия.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>АВИСМЕД, ООО ЛДЦ</t>
+          <t>А-КЛИНИК, ООО</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>5406513676</t>
+          <t>7203547497</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -6666,37 +7568,37 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>дерматология, косметология</t>
+          <t>терапия, дерматология, хирургия, гинекология, урология, эндокринология, онкодерматология</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Лечебно-диагностический центр «АвисМед», специалисты: гинеколог, дерматолог, косметолог, невролог, онколог, оториноларинголог, педиатр, стоматолог, терапевт, уролог, флеболог, хирург</t>
+          <t>Лицензия на медицинскую деятельность, прием врачей различных специальностей, медицинские услуги в прайсе.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+          <t>А-КЛИНИК, ООО</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1653000230</t>
+          <t>7203547497</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -6711,27 +7613,27 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
+          <t>терапия, дерматология, дерматоонкология, амбулаторная хирургия, маммология, проктология, гинекология, урология, эндокринология</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Услуги: Эндокринолог, Гастроэнтеролог, Гинеколог, Дерматолог, Кардиолог, Невролог, Онколог, Офтальмолог, Педиатр, Психотерапевт, Терапевт, Уролог, Флеболог, Хирург</t>
+          <t>Номер лицензии: Дневной стационар, терапия, дерматология, дерматоонкология, амбулаторная хирургия</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+          <t>А-МЦ УЛЬТРАМЕД, ООО</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>5406137478</t>
+          <t>5256051451</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -6746,37 +7648,37 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>управляющая компания сети клиник</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, терапия, урология, онкология, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
+          <t>акушерство и гинекология, гастроэнтерология, дерматология, кардиология, неврология, онкология, оториноларингология, пульмонология, ревматология, терапия, урология, эндокринология</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Направления деятельности</t>
+          <t>Прием врача-гинеколога, Прием врача-гастроэнтеролога, Прием врача-дерматолога / дерматовенеролога, Прием врача-кардиолога, Прием врача-невролога, Прием врача-онколога, Лечение ЛОР-заболеваний, Пульмонология, Прием врача-ревматолога, Прием врача-терапевта, Прием врача-уролога, Прием врача-эндокриноло</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, ООО</t>
+          <t>А-МЦ УЛЬТРАМЕД, ООО</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>7204082420</t>
+          <t>5256051451</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -6786,57 +7688,1217 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>управляющая компания сети клиник</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>аллергология, гинекология</t>
+          <t>акушерство и гинекология, гастроэнтерология, генетика, гепатология, дерматовенерология, кардиология, колопроктология, маммология, мануальная терапия, неврология, онкология, оториноларингология, пульмонология, ревматология, терапия, урология, эндокринология, функциональная диагностика</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности</t>
+          <t>Многопрофильный медицинский центр «Ультрамед» | Опытные врачи, широкий спектр медицинских услуг, все виды исследований в Нижнем Новгороде</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>А2МЕД ЧЕЛЯБИНСК, ООО</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>7451374192</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, терапия, урология, эндокринология</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Миссия клиники Парк Мед заключается в восстановлении и сохранении здоровья, используя современный медицинские технологии, профессионализм, заботу и доверие.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>А2МЕД ЧЕЛЯБИНСК, ООО</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>7451374192</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, терапия, урология, эндокринология</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Медицинский центр «ПаркМед» | Услуги медицинского центра «ПаркМед» | Специалисты клиники «ПаркМед» | Режим работы в праздничные дни в 2023 году | г. Челябинск, Краснопольский пр-т д.15Б</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>А2МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>6317157682</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>стоматология</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>А2МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>6317157682</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>стоматология</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>АВ ДГТУ, ООО</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>6165200482</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>дерматология, венерология</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Дерматовенеролог, дерматовенерология в профиле врачей и направлениях</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>АВ ДГТУ, ООО</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>6165200482</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, дерматовенерология, кардиология, неврология, оториноларинология, офтальмология, терапия, урология, функциональная диагностика, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Поликлиника «АвеВита» в Ростове-на-Дону на ул. Текучёва, 145</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>АВА-КАЗАНЬ, АО</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>1655146267</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, кардиология, неврология, онкология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, стоматология, косметология</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Услуги: Гинекология, Кардиология, Неврология, Онкология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стоматология, Косметология</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>АВА-КАЗАНЬ, АО</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>1655146267</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, педиатрия, диагностика, гематология, кардиология, неврология, онкология, маммология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, пластическая хирургия, косметология</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Клиника внимательной медицины 'Скандинавия'. Записаться на консультацию по номеру 8 (843) 200-10-65 круглосуточно.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>АВАНТА-МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>5406302509</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, урология, дерматология, отоларингология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, косметология, стоматология</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>АВАНТА-МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>5406302509</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, урология, отоларингология, дерматовенерология, дерматология, подология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, педиатрия, стоматология</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>АВАНТИС, ООО</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>5402038349</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>ортодонтия</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>АВАНТИС, ООО</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>5402038349</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>ортодонтия, терапия, хирургия, имплантация</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>6658006884</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>стоматология</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>6658006884</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>стоматология</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>5406513676</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>дерматология, косметология</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Лечебно-диагностический центр «АвисМед», специалисты: гинеколог, дерматолог, косметолог, невролог, онколог, оториноларинголог, педиатр, стоматолог, терапевт, уролог, флеболог, хирург</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>5406513676</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, дерматология, косметология, неврология, онкология, оториноларингология, педиатрия, стоматология, терапия, урология, флебология, хирургия</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Записаться на услуги лечебно-диагностического центра «АвисМед»</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>1653000230</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Услуги: Эндокринолог, Гастроэнтеролог, Гинеколог, Дерматолог, Кардиолог, Невролог, Онколог, Офтальмолог, Педиатр, Психотерапевт, Терапевт, Уролог, Флеболог, Хирург</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>1653000230</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>5406137478</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, терапия, урология, онкология, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Направления деятельности</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>5406137478</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, лечение бесплодия (ЭКО), общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, лучевая диагностика, терапия, урология, ультразвуковая диагностика, стоматология, онкология, восстановительное лечение, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Медицинский центр 'АВИЦЕННА' - частная клиника мирового уровня в Новосибирске</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>АВИЦЕННА, ООО</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>7204082420</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>аллергология, гинекология</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>АВИЦЕННА, ООО</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>7204082420</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>аллергология-иммунология, акушерство-гинекология, гастроэнтерология, дерматовенерология, кардиология, неврология, отоларингология, офтальмология, пульмонология, ревматология, стоматология, терапия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>5407494063</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>косметология, пластическая хирургия</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Лицензия №1, Приложение к лицензии №1, Приложение к лицензии №2-1, Приложение к лицензии №2-2, Приложение к лицензии №2-3, Лицензия №2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>5407494063</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>пластическая хирургия, врачебная косметология, диетология, сомнология</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>АГК, ООО</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>2461016768</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>llm7</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>медорганизация</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>не определено</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>гинекология, урология, хирургия, онкология, терапия</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Услуги центра: Акушерство и гинекология, Андрология и Урология, Хирургия, Маммология и онкология, Терапевт</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>АГК, ООО</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>2461016768</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>акушерство и гинекология, андрология и урология, лабораторная диагностика, физиотерапия, ультразвуковая диагностика, хирургия, сосудистая хирургия, оперативная гинекология, проктология, эндоскопия, маммология и онкология, терапия</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>ООО 'АГК' - первая частная клиника в Красноярске, занимающаяся вопросами мужского и женского здоровья с 1997г. Клиника лицензирована и соответствует всем требованиям медицинской безопасности.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>общая практика, дерматология, стоматология</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>6314040975</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>общая практика, дерматология, стоматология</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>6314040975</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
         </is>
       </c>
     </row>
@@ -7087,24 +9149,66 @@
           <t>Уфа</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>xn--b1aaegg8akarn3job.xn--p1ai</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 0278947517 найден на сайте</t>
+        </is>
+      </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr"/>
-      <c r="U2" s="2" t="inlineStr"/>
-      <c r="V2" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Прием (осмотр, консультация) врача-косметолога первичный»</t>
+        </is>
+      </c>
       <c r="W2" s="2" t="inlineStr"/>
-      <c r="X2" s="2" t="inlineStr"/>
-      <c r="Y2" s="2" t="inlineStr"/>
-      <c r="Z2" s="2" t="inlineStr"/>
-      <c r="AA2" s="2" t="inlineStr"/>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>похож</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>Цитологическое исследование микропрепарата кожи; Патолого-анатомическое исследование биопсийного (операционного) материала кожи; Биопсия кожи; Соскоб кожи; Инъекционное введение лекарственных препаратов в очаг поражения кожи; Очищение кожи лица и шеи; Вапоризация кожи лица; Удаление камедонов кожи; Удаление милиумов кожи; Удаление контагиозных моллюсков; Удаление ногтевых пластинок; Удаление ногтевой пластинки при помощи лазера; Удаление ксантелазм век; Ультразвуковое лечение кожи; Лазерная деструкция ткани кожи; Биопсия молочной железы чрескожная; Удаление атеромы; Удаление доброкачественных новообразований кожи; Удаление доброкачественных новообразований кожи методом электрокоагуляции; Удаление доброкачественных новообразований подкожно-жировой клетчатки; Вскрытие инфильтрата (угревого элемента) кожи и подкожно-жировой клетчатки; Прием (осмотр, консультация) врача-онколога первичный</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>гинеколог, дерматовенеролог, косметолог, онколог, терапевт, хирург</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -7167,24 +9271,62 @@
           <t>Пермь</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>stomatolorica.ru</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 5905280410 найден на сайте</t>
+        </is>
+      </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr"/>
-      <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W3" s="2" t="inlineStr"/>
-      <c r="X3" s="2" t="inlineStr"/>
-      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z3" s="2" t="inlineStr"/>
-      <c r="AA3" s="2" t="inlineStr"/>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>стоматолог</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -7248,7 +9390,9 @@
       <c r="Y4" s="2" t="inlineStr"/>
       <c r="Z4" s="2" t="inlineStr"/>
       <c r="AA4" s="2" t="inlineStr"/>
-      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -7295,24 +9439,66 @@
           <t>Нижний Новгород</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>8-nn.ru</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 5260143507 найден на сайте</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Документы оформляются на бланках установленного образца. Все филиалы имеют государственную лицензию на осуществление медицинской деятельности» (https://8-nn.ru)</t>
+        </is>
+      </c>
       <c r="W5" s="2" t="inlineStr"/>
-      <c r="X5" s="2" t="inlineStr"/>
-      <c r="Y5" s="2" t="inlineStr"/>
-      <c r="Z5" s="2" t="inlineStr"/>
-      <c r="AA5" s="2" t="inlineStr"/>
-      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>похож</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>Остроконечные кондиломы: d до 0,5 см; Остроконечные кондиломы: d более 0,5 см; Остроконечные кондиломы: удаление более 30 единиц; Анестезия ( местное обезболивание); Папиллома вульвы последующие; Папиллома шейки матки, последующие единицы; Папиллома вульвы, первая единица; Папиллома вульвы, последующие единицы; Папиллома шейки матки, первая единица; Радиоволновая конизация шейки матки; Радиоволновая биопсия шейки матки; Радиоволновая деструкция шейки матки; Удаление 1новообразования шейки матки,влагалища, вульвы до 0,5см; Удаление 1 новообразования шейки матки,влагалища,вульвы более 0,5см; Вакцинация от трихомониаза и бак. Вагиноза</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматовенеролог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, стоматолог, терапевт, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="AB5" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -7467,24 +9653,62 @@
           <t>Тюмень</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>a-clinik.ru</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 7203547497 найден на сайте</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="inlineStr"/>
-      <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W7" s="2" t="inlineStr"/>
-      <c r="X7" s="2" t="inlineStr"/>
-      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z7" s="2" t="inlineStr"/>
-      <c r="AA7" s="2" t="inlineStr"/>
-      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>гинеколог, дерматолог, косметолог, онкодерматолог, онколог, терапевт, уролог, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="AB7" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -7548,7 +9772,9 @@
       <c r="Y8" s="2" t="inlineStr"/>
       <c r="Z8" s="2" t="inlineStr"/>
       <c r="AA8" s="2" t="inlineStr"/>
-      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -7724,7 +9950,9 @@
       <c r="Y10" s="2" t="inlineStr"/>
       <c r="Z10" s="2" t="inlineStr"/>
       <c r="AA10" s="2" t="inlineStr"/>
-      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AB10" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -7796,7 +10024,9 @@
       <c r="Y11" s="2" t="inlineStr"/>
       <c r="Z11" s="2" t="inlineStr"/>
       <c r="AA11" s="2" t="inlineStr"/>
-      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -7860,7 +10090,9 @@
       <c r="Y12" s="2" t="inlineStr"/>
       <c r="Z12" s="2" t="inlineStr"/>
       <c r="AA12" s="2" t="inlineStr"/>
-      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AB12" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -8011,24 +10243,62 @@
           <t>Самара</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>a2med-stomat.ru</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Самара (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="inlineStr"/>
-      <c r="V14" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Медицинская деятельность осуществляется на основании лицензии №ЛО41-01184-63.00383779 от 11.07.2019, выданной Министерством здравоохранения Самарской области» (https://a2med-stomat.ru)</t>
+        </is>
+      </c>
       <c r="W14" s="2" t="inlineStr"/>
-      <c r="X14" s="2" t="inlineStr"/>
-      <c r="Y14" s="2" t="inlineStr"/>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z14" s="2" t="inlineStr"/>
-      <c r="AA14" s="2" t="inlineStr"/>
-      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>стоматолог, терапевт, хирург</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -8092,7 +10362,9 @@
       <c r="Y15" s="2" t="inlineStr"/>
       <c r="Z15" s="2" t="inlineStr"/>
       <c r="AA15" s="2" t="inlineStr"/>
-      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AB15" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -8247,28 +10519,62 @@
           <t>Казань</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>ava-kazan.ru</t>
+        </is>
+      </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились (гибко)</t>
-        </is>
-      </c>
-      <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Казань (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T17" s="2" t="inlineStr"/>
-      <c r="U17" s="2" t="inlineStr"/>
-      <c r="V17" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>приём врача в прайсе: «Прием (осмотр, консультация) аллерголога-иммунолога повторный (ДЕТСКИЙ ПРИЕМ)»</t>
+        </is>
+      </c>
       <c r="W17" s="2" t="inlineStr"/>
-      <c r="X17" s="2" t="inlineStr"/>
-      <c r="Y17" s="2" t="inlineStr"/>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z17" s="2" t="inlineStr"/>
-      <c r="AA17" s="2" t="inlineStr"/>
-      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматовенеролог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, ревматолог, терапевт, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -8544,7 +10850,9 @@
       <c r="Y20" s="2" t="inlineStr"/>
       <c r="Z20" s="2" t="inlineStr"/>
       <c r="AA20" s="2" t="inlineStr"/>
-      <c r="AB20" s="2" t="inlineStr"/>
+      <c r="AB20" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -8624,7 +10932,9 @@
       <c r="Y21" s="2" t="inlineStr"/>
       <c r="Z21" s="2" t="inlineStr"/>
       <c r="AA21" s="2" t="inlineStr"/>
-      <c r="AB21" s="2" t="inlineStr"/>
+      <c r="AB21" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -8688,7 +10998,9 @@
       <c r="Y22" s="2" t="inlineStr"/>
       <c r="Z22" s="2" t="inlineStr"/>
       <c r="AA22" s="2" t="inlineStr"/>
-      <c r="AB22" s="2" t="inlineStr"/>
+      <c r="AB22" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -8752,7 +11064,9 @@
       <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="2" t="inlineStr"/>
       <c r="AA23" s="2" t="inlineStr"/>
-      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AB23" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -9352,7 +11666,9 @@
       <c r="Y29" s="2" t="inlineStr"/>
       <c r="Z29" s="2" t="inlineStr"/>
       <c r="AA29" s="2" t="inlineStr"/>
-      <c r="AB29" s="2" t="inlineStr"/>
+      <c r="AB29" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -9416,7 +11732,9 @@
       <c r="Y30" s="2" t="inlineStr"/>
       <c r="Z30" s="2" t="inlineStr"/>
       <c r="AA30" s="2" t="inlineStr"/>
-      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AB30" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -9488,7 +11806,9 @@
       <c r="Y31" s="2" t="inlineStr"/>
       <c r="Z31" s="2" t="inlineStr"/>
       <c r="AA31" s="2" t="inlineStr"/>
-      <c r="AB31" s="2" t="inlineStr"/>
+      <c r="AB31" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -9535,13 +11855,29 @@
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr"/>
-      <c r="P32" s="2" t="inlineStr"/>
-      <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>avtokom54.ru</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Новосибирск (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="T32" s="2" t="inlineStr"/>
@@ -9552,7 +11888,9 @@
       <c r="Y32" s="2" t="inlineStr"/>
       <c r="Z32" s="2" t="inlineStr"/>
       <c r="AA32" s="2" t="inlineStr"/>
-      <c r="AB32" s="2" t="inlineStr"/>
+      <c r="AB32" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -9599,24 +11937,66 @@
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>avtor-e.ru</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 5407494063 найден на сайте</t>
+        </is>
+      </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T33" s="2" t="inlineStr"/>
-      <c r="U33" s="2" t="inlineStr"/>
-      <c r="V33" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W33" s="2" t="inlineStr"/>
-      <c r="X33" s="2" t="inlineStr"/>
-      <c r="Y33" s="2" t="inlineStr"/>
-      <c r="Z33" s="2" t="inlineStr"/>
-      <c r="AA33" s="2" t="inlineStr"/>
-      <c r="AB33" s="2" t="inlineStr"/>
+      <c r="X33" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z33" s="2" t="inlineStr">
+        <is>
+          <t>ELDERMAFILL HTL-T ampoule - Липомоделирующий лосьон для контуров лица и тела (5,0 мл.); ELDERMAFILL V-up gravitation ampoule - Аnti-age лосьон с полинуклеотидами для обновления структуры кожи лица и тела. Оказывает антигравитационные действия (5,0 мл.); HAIR X — Мезораствор для волос (4,0 мл.); Блефаропластика нижних век кожная с удалением грыж; Липомоделирование (всё тело)</t>
+        </is>
+      </c>
+      <c r="AA33" s="2" t="inlineStr">
+        <is>
+          <t>дерматолог, косметолог, психотерапевт, терапевт, трихолог, хирург</t>
+        </is>
+      </c>
+      <c r="AB33" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -9680,7 +12060,9 @@
       <c r="Y34" s="2" t="inlineStr"/>
       <c r="Z34" s="2" t="inlineStr"/>
       <c r="AA34" s="2" t="inlineStr"/>
-      <c r="AB34" s="2" t="inlineStr"/>
+      <c r="AB34" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -9744,7 +12126,9 @@
       <c r="Y35" s="2" t="inlineStr"/>
       <c r="Z35" s="2" t="inlineStr"/>
       <c r="AA35" s="2" t="inlineStr"/>
-      <c r="AB35" s="2" t="inlineStr"/>
+      <c r="AB35" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -9808,7 +12192,9 @@
       <c r="Y36" s="2" t="inlineStr"/>
       <c r="Z36" s="2" t="inlineStr"/>
       <c r="AA36" s="2" t="inlineStr"/>
-      <c r="AB36" s="2" t="inlineStr"/>
+      <c r="AB36" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -9872,7 +12258,9 @@
       <c r="Y37" s="2" t="inlineStr"/>
       <c r="Z37" s="2" t="inlineStr"/>
       <c r="AA37" s="2" t="inlineStr"/>
-      <c r="AB37" s="2" t="inlineStr"/>
+      <c r="AB37" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -10064,7 +12452,9 @@
       <c r="Y39" s="2" t="inlineStr"/>
       <c r="Z39" s="2" t="inlineStr"/>
       <c r="AA39" s="2" t="inlineStr"/>
-      <c r="AB39" s="2" t="inlineStr"/>
+      <c r="AB39" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -10111,24 +12501,66 @@
           <t>Самара</t>
         </is>
       </c>
-      <c r="O40" s="2" t="inlineStr"/>
-      <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="2" t="inlineStr"/>
-      <c r="R40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>azbuka-samara.ru</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Самара (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T40" s="2" t="inlineStr"/>
-      <c r="U40" s="2" t="inlineStr"/>
-      <c r="V40" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V40" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W40" s="2" t="inlineStr"/>
-      <c r="X40" s="2" t="inlineStr"/>
-      <c r="Y40" s="2" t="inlineStr"/>
-      <c r="Z40" s="2" t="inlineStr"/>
-      <c r="AA40" s="2" t="inlineStr"/>
-      <c r="AB40" s="2" t="inlineStr"/>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>Анестезия</t>
+        </is>
+      </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтеролог, дерматолог, невролог, отоларинголог, офтальмолог, педиатр, стоматолог, терапевт, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="AB40" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -10175,24 +12607,66 @@
           <t>Самара</t>
         </is>
       </c>
-      <c r="O41" s="2" t="inlineStr"/>
-      <c r="P41" s="2" t="inlineStr"/>
-      <c r="Q41" s="2" t="inlineStr"/>
-      <c r="R41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>azbuka-samara.ru</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Самара (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T41" s="2" t="inlineStr"/>
-      <c r="U41" s="2" t="inlineStr"/>
-      <c r="V41" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V41" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W41" s="2" t="inlineStr"/>
-      <c r="X41" s="2" t="inlineStr"/>
-      <c r="Y41" s="2" t="inlineStr"/>
-      <c r="Z41" s="2" t="inlineStr"/>
-      <c r="AA41" s="2" t="inlineStr"/>
-      <c r="AB41" s="2" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>Анестезия</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтеролог, дерматолог, невролог, отоларинголог, офтальмолог, педиатр, стоматолог, терапевт, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="AB41" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test-40: конвейер 2026-08-27 (run 33099264784)
</commit_message>
<xml_diff>
--- a/output/Тест40_2026-08-27.xlsx
+++ b/output/Тест40_2026-08-27.xlsx
@@ -1521,22 +1521,46 @@
       <c r="G15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>vesna24.ru</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>косметолог, онколог, хирург</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>единогласно мед (реестр + 3 судьи)</t>
         </is>
       </c>
     </row>
@@ -1872,22 +1896,46 @@
       <c r="G20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>venum-center.ru</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Лицензия № Л041-01107-72/00361525» (https://venum-center.ru)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>флеболог, хирург</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>единогласно мед (реестр + 3 судьи)</t>
         </is>
       </c>
     </row>
@@ -1970,7 +2018,7 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>единогласно мед (реестр + 2 судьи)</t>
+          <t>единогласно мед (реестр + 3 судьи)</t>
         </is>
       </c>
     </row>
@@ -2006,22 +2054,42 @@
       <c r="G22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>grandavenue.ru</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>медицинских признаков на сайте нет: ни лицензии, ни врачей, ни приёмов (https://grandavenue.ru)</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>РАСХОЖДЕНИЕ: реестр мед, судьи мед 0/3 — на ручную</t>
         </is>
       </c>
     </row>
@@ -2558,22 +2626,42 @@
       <c r="G30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>avr-rostov.ru</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>РАСХОЖДЕНИЕ: реестр мед, судьи мед 0/3 — на ручную</t>
         </is>
       </c>
     </row>
@@ -2818,15 +2906,23 @@
       <c r="G34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>avtotranskontejner.clients.site</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr"/>
@@ -2920,22 +3016,46 @@
       <c r="G36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>mc-semya.ru</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, оториноларинголог, офтальмолог, педиатр, пульмонолог, ревматолог, терапевт, трихолог, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr"/>
       <c r="P36" s="2" t="inlineStr"/>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>единогласно мед (реестр + 3 судьи)</t>
         </is>
       </c>
     </row>
@@ -3105,22 +3225,46 @@
       <c r="G39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
-      <c r="M39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>«…/news/cherno-belaya-vecherinka-kommersant-sibir-shakhmaty-klassika-i-zabota-o-zdorove-ot-kliniki-smitra/)  [![Image 57: Сеть клиник «Смитра» признана лучшей в здравоохранении на городском конкурсе](https://smitra.ru/upload/webp/upload/iblock/f1d/79x9y5vtvwfiecyksen2q2yv5k2aiqpa.webp)](https://smitra.ru/news/set-klinik-smitra-priznana-luchshey-v-zdravookhranenii-na-goro…» (https://smitra.ru)</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уролог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr"/>
       <c r="P39" s="2" t="inlineStr"/>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>единогласно мед (реестр + 3 судьи)</t>
         </is>
       </c>
     </row>
@@ -5891,7 +6035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6788,24 +6932,110 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>АБВ+, ООО</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2465176508</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>vesna24.ru</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: vesna24.ru (страниц скачано: 5)
+TITLE: Косметология VESNA в Красноярске, клиника эстетической медицины
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://vesna24.ru:
+    «## Лицензированная клиника в Красноярске»
+    «*    Лицензия Л041-01019-24/00338199 от 13.09.2018 г.(действует бессрочно), выдана Министерством здравоохранения Красноярского края»
+    «*   ИНН 2465176508»
+    «*   ОГРН 1182468003497»
+    «*    Адрес оказания мед. услуг: 660077, Красноярский край, город Красноярск, улица Молокова, дом 15, помещение 42, этаж 1»
+  https://vesna24.ru/prices:
+    «*    Лицензия Л041-01019-24/00338199 от 13.09.2018 г.(действует бессрочно), выдана Министерством здравоохранения Красноярского края»
+    «*   ИНН 2465176508»
+    «*   ОГРН 1182468003497»
+    «*    Адрес оказания мед. услуг: 660077, Красноярский край, город Красноярск, улица Молокова, дом 15, помещение 42, этаж 1»
+  https://vesna24.ru/services:
+    «*    Лицензия Л041-01019-24/00338199 от 13.09.2018 г.(действует бессрочно), выдана Министерством здравоохранения Красноярского края»
+    «*   ИНН 2465176508»
+    «*   ОГРН 1182468003497»
+    «*    Адрес оказания мед. услуг: 660077, Красноярский край, город Красноярск, улица Молокова, дом 15, помещение 42, этаж 1»
+  https://vesna24.ru/services/botox:
+    «*    Лицензия Л041-01019-24/00338199 от 13.09.2018 г.(действует бессрочно), выдана Министерством здравоохранения Красноярского края»
+    «*   ИНН 2465176508»
+    «*   ОГРН 1182468003497»
+    «*    Адрес оказания мед. услуг: 660077, Красноярский край, город Красноярск, улица Молокова, дом 15, помещение 42, этаж 1»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): косметолог, онколог, хирург
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: косметолог, косметология
+ЛИЦЕНЗИЯ (строка с сайта): «Лицензированная клиника в Красноярске» (https://vesna24.ru)
+ПОЗИЦИИ ПРАЙСА (первые 30 из 56):
+  опытных врачей-косметологов — 3 199 ₽
+  Мы свяжемся с вами для записи и предоставим скидку — 1000₽
+  Скидка — 1000₽
+  Межбровье — 3 590₽
+  Уголки глаз — 3 590₽
+  Лоб + межбровье — 6 990₽
+  Межбровье + глаза — 6 990₽
+  Лоб + межбровье + глаза — 9 990₽
+  Биоревитализация NCTF 135 + пилинг — 9 990₽
+  IPL фототерапия + биоревитализация NCTF — 135 9 990₽
+  IPL фототерапия + пилинг + биоревитализация NCTF 1 — 35 11 990₽
+  Коктейль Монако (Диспорт + NCTF 135) — 11 990₽
+  PDRN (Bellarti Nucleo) + Экзосомы — 21 990₽
+  RF лифтинг лицо + экзосомы — 19 990₽
+  RF лифтинг лицо + шея + экзосомы — 27 990₽
+  RF лифтинг + PDRN (Bellarti Nucleo) — 24 990₽
+  Бионутрилифт (ArtFiller + NCTF 135) — 24 990₽
+  Фототерапия крылья носа — 2 990₽
+  Фототерапия подбородок — 2 990₽
+  Фототерапия лоб — 3 990₽
+  Фототерапия щеки — 5 990₽
+  Фототерапия лица — 7 990₽
+  Фототерапия лицо + шея — 9 990₽
+  Фототерапия лицо + шея + декольте — 11 990₽
+  Феруловый Mediderma — 3 190₽
+  Азелаиновый Mediderma — 3 190₽
+  Салициловый Mediderma — 3 190₽
+  Ретиноловый Mediderma — 4 990₽
+  Пилинг Джесснера — 3 990₽
+  Классика — 990₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>6165200482</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>аве-вита.рф</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>САЙТ: аве-вита.рф (страниц скачано: 3)
 TITLE: Поликлиника «АвеВита» в Ростове-на-Дону
@@ -6850,26 +7080,26 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>1655146267</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>ava-kazan.ru</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>САЙТ: ava-kazan.ru (страниц скачано: 5)
 TITLE: Клиника внимательной медицины "Скандинавия"
@@ -6960,26 +7190,26 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="16">
+      <c r="A16" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>5406302509</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>avanta-med.ru</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avanta-med.ru (страниц скачано: 5)
 TITLE: Медицинский центр Аванта-Мед в Новосибирске
@@ -7035,26 +7265,26 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>АВАНТИС, ООО</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>5402038349</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>avantis-stom.ru</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avantis-stom.ru (страниц скачано: 1)
 TITLE: Брекеты в Новосибирске: цена на установку от 14900 рублей
@@ -7082,26 +7312,80 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>АВАТАР, ООО</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>7203314735</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>venum-center.ru</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: venum-center.ru (страниц скачано: 1)
+TITLE: Лечение варикоза в Тюмени | Флеболог в Тюмени | УЗИ вен ног в Тюмени | Центр лечения варикоза «Венум»
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://venum-center.ru:
+    «г. Тюмень, ул. Комсомольская, 8»
+    «### Процедура осуществляется при помощи инновационного оборудования, под УЗИ-контролем, что полностью исключает любые риски и ошибки.»
+    «г. Тюмень, ул. Комсомольская, д. 8»
+    «Режим работы: Пн-Пт с 10 до 20, Сб-Вс с 10 до 18»
+    «Лицензия № Л041-01107-72/00361525»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): флеболог, хирург
+ЛИЦЕНЗИЯ (строка с сайта): «Лицензия № Л041-01107-72/00361525» (https://venum-center.ru)
+ПОЗИЦИИ ПРАЙСА (первые 14 из 14):
+  Прием Флеболога + УЗИ вен в ПОДАРОК всего — 1600 руб.
+  Прием врача-флеболога первичный + УЗИ — 1600
+  Прием врача-флеболога первичный с готовым заключением из другой клиники (второе мнение) — 800
+  Лазерное лечение варикоза (ЭВЛК) перфоранта или притока (анализы бесплатно) — 14000
+  Лазерное лечение варикоза (ЭВЛК) одной вены V категории (анализы + 3 послеоперационных приема бесплатно) — 33000
+  Лазерное лечение варикоза (ЭВЛК) одной вены + минифлебэктомия притоков IV категории (анализы + компрессионный трикотаж + — 48000
+  Лазерное лечение варикоза (ЭВЛК) одной вены + склерооблитерация притоков III категории (анализы + компрессионный трикота — 56000
+  Лазерное лечение варикоза (ЭВЛК) одной вены + склерооблитерация + минифлебэктомия притоков II категории (анализы + компр — 62000
+  Лазерное лечение варикоза (ЭВЛК) одной вены (диаметром более 1 см) + склерооблитерация + минифлебэктомия I категории (ан — 70000
+  Лазерное лечение варикоза (ЭВЛК) с выраженными трофическими изменениями I+ категории (анализы + компрессионный трикотаж  — 75000
+  Склеротерапия (удаление сосудистых звездочек) введение одной ампулы склерозанта — 9000
+  Повторный прием после операции (3 приема в течение года бесплатные) — 500
+  Перевязка при трофической язве с использованием современного раневого покрытия — 300
+  Анализы без операции (без операции) — 2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>7203527116</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>medlogika.ru</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>САЙТ: medlogika.ru (страниц скачано: 5)
 TITLE: Медицинский центр "МедЛогика" - клиника с добрым сердцем в Тюмени
@@ -7199,26 +7483,64 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>АВЕНЮ, ООО</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>0278947838</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>grandavenue.ru</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: grandavenue.ru (страниц скачано: 1)
+TITLE: Жилой комплекс бизнес-класса для активной жизни в мегаполисе
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://grandavenue.ru:
+    «Уфа, ул. 50-летия Октября»
+    «Уфа, ул. 50-летия Октября»
+    «ул. Цюрупы, 30»
+    «ул. Рудольфа Нуреева, 5»
+ПОЗИЦИИ ПРАЙСА (первые 1 из 1):
+  Ежемесячный платёж — 50 000 руб</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>6658006884</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>aviodent.ru</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>САЙТ: aviodent.ru (страниц скачано: 2)
 TITLE: Сеть стоматологических клиник Доктора Мансурского | Платная стоматология в в Екатеринбурге
@@ -7250,26 +7572,26 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
+    <row r="22">
+      <c r="A22" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>5406513676</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>avismed-nsk.ru</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avismed-nsk.ru (страниц скачано: 5)
 TITLE: Лечебно-диагностический центр «АвисМед»
@@ -7316,26 +7638,26 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+    <row r="23">
+      <c r="A23" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>1653000230</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>avicenna-endocrin.ru</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna-endocrin.ru (страниц скачано: 5)
 TITLE: Клиника профессора Анчиковой - Главная
@@ -7395,26 +7717,26 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>5406137478</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>avicenna-nsk.ru</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna-nsk.ru (страниц скачано: 4)
 TITLE: Медицинский центр "АВИЦЕННА" - частная клиника мирового уровня в Новосибирске
@@ -7446,26 +7768,26 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
+    <row r="25">
+      <c r="A25" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>7204082420</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>avicenna72.ru</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna72.ru (страниц скачано: 5)
 TITLE: Многопрофильный медицинский центр в Тюмени — «Авиценна»
@@ -7572,26 +7894,26 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
+    <row r="26">
+      <c r="A26" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>АВК-МЕД, ООО</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>5260156369</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>avk-med.inni.info</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avk-med.inni.info (страниц скачано: 5)
 TITLE: ООО «АВК-Мед»
@@ -7645,26 +7967,80 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>АВРОРА, ООО</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>6164209193</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>avr-rostov.ru</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: avr-rostov.ru (страниц скачано: 4)
+TITLE: Купить автомобиль в Ростове-на-Дону - автосалон Аврора
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://avr-rostov.ru:
+    «г. Ростов-на-Дону, проспект Шолохова, 247»
+    «г. Ростов-на-Дону, проспект Шолохова, 247»
+    «Режим работы»
+    «г. Ростов-на-Дону, проспект Шолохова, 247»
+    «Режим работы»
+    «Банк-партнер: ВТБ (ПАО), Лицензия Банка ВТБ — №1000 от 08.07.2015. Партнер по страхованию: СПАО «Ингосстрах», лицензия ЦБ РФ № 0928»
+    «Реквизиты организации: ООО "АВРОРА" ИНН 9705237502 ОГРН 1257700028068»
+  https://avr-rostov.ru/contact:
+    «г. Ростов-на-Дону, проспект Шолохова, 247»
+    «г. Ростов-на-Дону, проспект Шолохова, 247»
+    «Режим работы»
+    «г. Ростов-на-Дону, проспект Шолохова, 247»
+    «Режим работы»
+    «г. Ростов-на-Дону, проспект Шолохова, 247»
+    «Режим работы»
+    «Банк-партнер: ВТБ (ПАО), Лицензия Банка ВТБ — №1000 от 08.07.2015. Партнер по страхованию: СПАО «Ингосстрах», лицензия ЦБ РФ № 0928»
+    «Реквизиты организации: ООО "АВРОРА" ИНН 9705237502 ОГРН 1257700028068»
+ЛИЦЕНЗИЯ (строка с сайта): «Для получения подробной информации о стоимости автомобилей обращайтесь к менеджерам по продажам. Любая информация, содержащаяся на настоящем сайте, носит исключительно справочный характер и ни при как» (https://avr-rostov.ru)
+ПОЗИЦИИ ПРАЙСА (первые 3 из 3):
+  в кредит — 24 579 ₽
+  ✔ Доп. скидка до — 300 000₽
+  Оставьте заявку и получите скидку — 30 000₽</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>АВТО-МЕД, ООО</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>6324110942</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>флеболог-тольятти.рф</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>САЙТ: флеболог-тольятти.рф (страниц скачано: 1)
 TITLE: Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.!
@@ -7681,26 +8057,26 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
+    <row r="29">
+      <c r="A29" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>5407494063</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>avtor-e.ru</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avtor-e.ru (страниц скачано: 5)
 TITLE: Клиника врачебной косметологии в Новосибирске | Услуги пластической хирургии в авторской клинике доктора Егорова
@@ -7774,26 +8150,78 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>АГАТ, ООО</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>6162081830</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>mc-semya.ru</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: mc-semya.ru (страниц скачано: 5)
+TITLE: Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение.
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://mc-semya.ru:
+    «[О клинике](https://mc-semya.ru/about/)[Отзывы](https://mc-semya.ru/reviews/)[Новости](https://mc-semya.ru/media/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)»
+    «Из центра Ростова-на-Дону до медицинского центра "Семья" на ул. Дачной можно доехать автобусами № 1, 17, 17а, 27, 43, 44, 49, 83 и 99.»
+    «До филиала МЦ "Семья" на Будённовском проспекте удобно добираться автобусами № 17, 17а, 33, 40, 43, 55, 65, 65а, 78, 83 85а, 92 и 99.»
+    «*   **Адрес:** Ростов-на-Дону, медицинский центр «Семья», ул. Дачная, 8; пр-кт Буденновский, 61/12.»
+    «[Пациентам](https://mc-semya.ru/pravovaya-informatsiya/patients/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)[Контакты](https://mc-semya.ru/contacts/)»
+  https://mc-semya.ru/uslugi:
+    «[О клинике](https://mc-semya.ru/about/)[Отзывы](https://mc-semya.ru/reviews/)[Новости](https://mc-semya.ru/media/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)»
+    «[Пациентам](https://mc-semya.ru/pravovaya-informatsiya/patients/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)[Контакты](https://mc-semya.ru/contacts/)»
+  https://mc-semya.ru/uslugi/allergologiya-immunologiya:
+    «[О клинике](https://mc-semya.ru/about/)[Отзывы](https://mc-semya.ru/reviews/)[Новости](https://mc-semya.ru/media/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)»
+    «[Пациентам](https://mc-semya.ru/pravovaya-informatsiya/patients/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)[Контакты](https://mc-semya.ru/contacts/)»
+  https://mc-semya.ru/uslugi/allergologiya-immunologiya/lechenie-allergii-asit:
+    «[О клинике](https://mc-semya.ru/about/)[Отзывы](https://mc-semya.ru/reviews/)[Новости](https://mc-semya.ru/media/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)»
+    «[Пациентам](https://mc-semya.ru/pravovaya-informatsiya/patients/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)[Контакты](https://mc-semya.ru/contacts/)»
+  https://mc-semya.ru/uslugi/anesteziologiya-i-reanimatsiya:
+    «[О клинике](https://mc-semya.ru/about/)[Отзывы](https://mc-semya.ru/reviews/)[Новости](https://mc-semya.ru/media/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)»
+    «[Пациентам](https://mc-semya.ru/pravovaya-informatsiya/patients/)[Партнеры / Лицензии](https://mc-semya.ru/pravovaya-informatsiya/licenses/)[Карьера](https://mc-semya.ru/career/)[Контакты](https://mc-semya.ru/contacts/)»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, оториноларинголог, офтальмолог, педиатр, пульмонолог, ревматолог, терапевт, трихолог, уролог, флеболог, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, дерматология, косметолог, косметология, трихолог, трихология
+ЛИЦЕНЗИЯ (строка с сайта): «О клиникеОтзывыНовостиПартнеры / ЛицензииКарьера» (https://mc-semya.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>АГК, ООО</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>2461016768</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>agk24.ru</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>САЙТ: agk24.ru (страниц скачано: 5)
 TITLE: Вопросы женского и мужского здоровья | ООО "Андро-гинекологическая клиника", г. Красноярск
@@ -7839,26 +8267,125 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: smitra.ru (страниц скачано: 5)
+TITLE: Многопрофильные клиники «Смитра» в Новосибирске
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://smitra.ru:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/news/novaya-usluga-analiz-na-antitela-igm-k-khantavirusam:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/news/novaya-usluga-lechenie-i-omolozhenie-v-ginekologii-lazerom-so-bioxel:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/news/novaya-usluga-podbor-kontaktnykh-linz:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/patients/bonus/uslugi-s-povyshennym-bonusom:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уролог, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, косметолог, косметология, трихолог
+ЛИЦЕНЗИЯ (строка с сайта): «Лицензия» (https://smitra.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>7813610598</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>azbuka-samara.ru</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>САЙТ: azbuka-samara.ru (страниц скачано: 3)
 TITLE: Семейный медицинский центр Самара 🏥 | Детский развивающий клуб
@@ -7891,26 +8418,26 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
+    <row r="34">
+      <c r="A34" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>6314040975</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>azbuka-samara.ru</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>САЙТ: azbuka-samara.ru (страниц скачано: 3)
 TITLE: Семейный медицинский центр Самара 🏥 | Детский развивающий клуб
@@ -7954,7 +8481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9287,16 +9814,16 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>АВ ДГТУ, ООО</t>
+          <t>АБВ+, ООО</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>6165200482</t>
+          <t>2465176508</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -9316,27 +9843,27 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Гинекология, Дерматовенерология, Кардиология, Неврология, Оториноларинология, Офтальмология, Терапия, Урология, Функциональная диагностика, Хирургия, Эндокринология, Стоматология, Гастроэнтерология</t>
+          <t>косметология, онкология, хирургия</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>TITLE: Поликлиника «АвеВита» в Ростове-на-Дону</t>
+          <t>«Лицензия Л041-01019-24/00338199 от 13.09.2018 г., выдана Министерством здравоохранения Красноярского края»</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>АВ ДГТУ, ООО</t>
+          <t>АБВ+, ООО</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>6165200482</t>
+          <t>2465176508</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9356,27 +9883,27 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>дерматология, венерология</t>
+          <t>косметология</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Дерматовенеролог, дерматовенерология в профиле врачей и направлениях</t>
+          <t>Лицензия Л041-01019-24/00338199 от 13.09.2018 г.(действует бессрочно), выдана Министерством здравоохранения Красноярского края</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>АВ ДГТУ, ООО</t>
+          <t>АБВ+, ООО</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>6165200482</t>
+          <t>2465176508</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -9396,27 +9923,27 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>гинекология, дерматовенерология, кардиология, неврология, оториноларинология, офтальмология, терапия, урология, функциональная диагностика, хирургия, эндокринология</t>
+          <t>косметология</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Поликлиника «АвеВита» в Ростове-на-Дону на ул. Текучёва, 145</t>
+          <t>Лицензированная клиника в Красноярске</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>АВА-КАЗАНЬ, АО</t>
+          <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>1655146267</t>
+          <t>6165200482</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -9431,32 +9958,32 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Педиатрия, Диагностика, Гинекология, Оперативная гинекология, Ведение беременности, Гематология, Кардиология, Неврология, Онкология, Маммология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стационар, Чек‑апы, Детские чек‑апы, Роддом, Реанимация новорожденных, Пластическая хирургия, Косметология, ЭКО, Криоконсервация стволовых клеток из пуповинной крови</t>
+          <t>Гинекология, Дерматовенерология, Кардиология, Неврология, Оториноларинология, Офтальмология, Терапия, Урология, Функциональная диагностика, Хирургия, Эндокринология, Стоматология, Гастроэнтерология</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Гинекология | Оперативная гинекология | Ведение беременности | Гематология | Кардиология | Неврология | Онкология, маммология</t>
+          <t>TITLE: Поликлиника «АвеВита» в Ростове-на-Дону</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>АВА-КАЗАНЬ, АО</t>
+          <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1655146267</t>
+          <t>6165200482</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -9471,32 +9998,32 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>гинекология, кардиология, неврология, онкология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, стоматология, косметология</t>
+          <t>дерматология, венерология</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Услуги: Гинекология, Кардиология, Неврология, Онкология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стоматология, Косметология</t>
+          <t>Дерматовенеролог, дерматовенерология в профиле врачей и направлениях</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>АВА-КАЗАНЬ, АО</t>
+          <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1655146267</t>
+          <t>6165200482</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -9511,32 +10038,32 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>гинекология, педиатрия, диагностика, гематология, кардиология, неврология, онкология, маммология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, пластическая хирургия, косметология</t>
+          <t>гинекология, дерматовенерология, кардиология, неврология, оториноларинология, офтальмология, терапия, урология, функциональная диагностика, хирургия, эндокринология</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Клиника внимательной медицины 'Скандинавия'. Записаться на консультацию по номеру 8 (843) 200-10-65 круглосуточно.</t>
+          <t>Поликлиника «АвеВита» в Ростове-на-Дону на ул. Текучёва, 145</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>АВАНТА-МЕД, ООО</t>
+          <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>5406302509</t>
+          <t>1655146267</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -9556,27 +10083,27 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, дерматовенерология, дерматология, подология, отоларингология, сурдология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексуология, педиатрия, стоматология, косметология, диагностика</t>
+          <t>Педиатрия, Диагностика, Гинекология, Оперативная гинекология, Ведение беременности, Гематология, Кардиология, Неврология, Онкология, Маммология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стационар, Чек‑апы, Детские чек‑апы, Роддом, Реанимация новорожденных, Пластическая хирургия, Косметология, ЭКО, Криоконсервация стволовых клеток из пуповинной крови</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+          <t>Гинекология | Оперативная гинекология | Ведение беременности | Гематология | Кардиология | Неврология | Онкология, маммология</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>АВАНТА-МЕД, ООО</t>
+          <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>5406302509</t>
+          <t>1655146267</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -9596,27 +10123,27 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, дерматология, отоларингология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, косметология, стоматология</t>
+          <t>гинекология, кардиология, неврология, онкология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, стоматология, косметология</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+          <t>Услуги: Гинекология, Кардиология, Неврология, Онкология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стоматология, Косметология</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>АВАНТА-МЕД, ООО</t>
+          <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>5406302509</t>
+          <t>1655146267</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -9636,27 +10163,27 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, отоларингология, дерматовенерология, дерматология, подология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, педиатрия, стоматология</t>
+          <t>гинекология, педиатрия, диагностика, гематология, кардиология, неврология, онкология, маммология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, пластическая хирургия, косметология</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+          <t>Клиника внимательной медицины 'Скандинавия'. Записаться на консультацию по номеру 8 (843) 200-10-65 круглосуточно.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>АВАНТИС, ООО</t>
+          <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>5402038349</t>
+          <t>5406302509</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -9671,32 +10198,32 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>ортодонтия, терапия, хирургия, имплантация, профессиональная чистка, отбеливание, элайнеры</t>
+          <t>гинекология, урология, дерматовенерология, дерматология, подология, отоларингология, сурдология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексуология, педиатрия, стоматология, косметология, диагностика</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Первичная консультация ортодонта — 500 руб</t>
+          <t>Медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>АВАНТИС, ООО</t>
+          <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>5402038349</t>
+          <t>5406302509</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -9711,32 +10238,32 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>ортодонтия</t>
+          <t>гинекология, урология, дерматология, отоларингология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, косметология, стоматология</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
+          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>АВАНТИС, ООО</t>
+          <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>5402038349</t>
+          <t>5406302509</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -9751,32 +10278,32 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>ортодонтия, терапия, хирургия, имплантация</t>
+          <t>гинекология, урология, отоларингология, дерматовенерология, дерматология, подология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, педиатрия, стоматология</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
+          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ МЕД, ООО</t>
+          <t>АВАНТИС, ООО</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>7203527116</t>
+          <t>5402038349</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -9796,32 +10323,32 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология, ультразвуковая диагностика, функциональная диагностика, нутрициология, психология</t>
+          <t>ортодонтия, терапия, хирургия, имплантация, профессиональная чистка, отбеливание, элайнеры</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Гинеколог, врач УЗИ, детский гинеколог — 2 000 ₽</t>
+          <t>Первичная консультация ортодонта — 500 руб</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ МЕД, ООО</t>
+          <t>АВАНТИС, ООО</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>7203527116</t>
+          <t>5402038349</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -9836,32 +10363,32 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология</t>
+          <t>ортодонтия</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр 'МедЛогика' - клиника с добрым сердцем в Тюмени. Лицензии и сертификаты доступны на сайте. Указаны медицинские специалисты и услуги.</t>
+          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+          <t>АВАНТИС, ООО</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>6658006884</t>
+          <t>5402038349</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -9876,32 +10403,32 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>стоматология, детская стоматология, имплантация, протезирование, пародонтология, гигиена, хирургия, ортопедическая стоматология</t>
+          <t>ортодонтия, терапия, хирургия, имплантация</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн.</t>
+          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+          <t>АВАТАР, ООО</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>6658006884</t>
+          <t>7203314735</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -9911,37 +10438,37 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>стоматология</t>
+          <t>флебология, хирургия</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
+          <t>«Лицензия № Л041-01107-72/00361525»</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+          <t>АВАТАР, ООО</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>6658006884</t>
+          <t>7203314735</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -9951,37 +10478,37 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>стоматология</t>
+          <t>флебология</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
+          <t>Лицензия № Л041-01107-72/00361525 на медицинскую деятельность, приём врача-флеболога, медицинские услуги в прайсе</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>АВИСМЕД, ООО ЛДЦ</t>
+          <t>АВАТАР, ООО</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>5406513676</t>
+          <t>7203314735</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -9996,32 +10523,32 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Диагностическое отделение, Консультативное отделение, Косметологическое отделение, Педиатрическое отделение, Хирургическое отделение</t>
+          <t>флебология, хирургия</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Лечебно-диагностический центр «АвисМед»</t>
+          <t>Лицензия № Л041-01107-72/00361525, приём врача-флеболога, лазерное лечение варикоза, склеротерапия, перевязка при трофической язве</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>АВИСМЕД, ООО ЛДЦ</t>
+          <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>5406513676</t>
+          <t>7203527116</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -10031,37 +10558,37 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>дерматология, косметология</t>
+          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология, ультразвуковая диагностика, функциональная диагностика, нутрициология, психология</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Лечебно-диагностический центр «АвисМед», специалисты: гинеколог, дерматолог, косметолог, невролог, онколог, оториноларинголог, педиатр, стоматолог, терапевт, уролог, флеболог, хирург</t>
+          <t>Гинеколог, врач УЗИ, детский гинеколог — 2 000 ₽</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>АВИСМЕД, ООО ЛДЦ</t>
+          <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>5406513676</t>
+          <t>7203527116</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -10071,37 +10598,37 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>гинекология, дерматология, косметология, неврология, онкология, оториноларингология, педиатрия, стоматология, терапия, урология, флебология, хирургия</t>
+          <t>акушерство и гинекология, кардиология, неврология, терапия, гастроэнтерология, урология, хирургия, эндокринология, психология, nutriциология</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Записаться на услуги лечебно-диагностического центра «АвисМед»</t>
+          <t>2021 г. — "Акушерство и гинекология", Тюменский государственный медицинский университет</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+          <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>1653000230</t>
+          <t>7203527116</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -10116,152 +10643,140 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>эндокринология, детская эндокринология, кардиология, терапия, ультразвуковая диагностика, гастроэнтерология, детская гастроэнтерология, андрология‑урология, детская урология‑андрология, акушер‑гинекология, детская акушер‑гинекология, неврология, детская неврология, остеопатия, детская остеопатия, мануальная терапия, сосудистый хирург‑флебология, онкология, маммология, хирургия (включая ожоговый хирург), нефрология, детская нефрология, психотерапия, детская психотерапия, массаж, нутрициология, офтальмология, детская офтальмология, функциональная диагностика, травматология‑ортопедия, педиатрия, дерматология, детская дерматология, генетические исследования, криодеструкция, биоимпедансометрия, физиотерапия, озонотерапия, склеротерапия, краниосакральная терапия</t>
+          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
+          <t>Медицинский центр 'МедЛогика' - клиника с добрым сердцем в Тюмени. Лицензии и сертификаты доступны на сайте. Указаны медицинские специалисты и услуги.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+          <t>АВЕНЮ, ООО</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>1653000230</t>
+          <t>0278947838</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
-        </is>
-      </c>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Услуги: Эндокринолог, Гастроэнтеролог, Гинеколог, Дерматолог, Кардиолог, Невролог, Онколог, Офтальмолог, Педиатр, Психотерапевт, Терапевт, Уролог, Флеболог, Хирург</t>
+          <t>Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+          <t>АВЕНЮ, ООО</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>1653000230</t>
+          <t>0278947838</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
-        </is>
-      </c>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
+          <t>TITLE: Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+          <t>АВЕНЮ, ООО</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>5406137478</t>
+          <t>0278947838</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>гинекология, кардиология и сердечно‑сосудистая хирургия, неврология и нейрохирургия, травматология и ортопедия, урология, онкология, оториноларингология, офтальмология и микрохирургия глаза, пластическая и реконструктивная хирургия, педиатрия, терапия, стоматология, лечения бесплодия (ЭКО), лабораторная и генетическая диагностика, лучевая диагностика, восстановительное лечение</t>
-        </is>
-      </c>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>TITLE: Медицинский центр "АВИЦЕННА" - частная клиника мирового уровня в Новосибирске; меню сайта содержит разделы «Клиника гинекологическое», «Клиника кардиологии», «Клиника неврологии», «Клиника онкологии» и др., а также ссылки «Лицензии».</t>
+          <t>Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>5406137478</t>
+          <t>6658006884</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -10276,32 +10791,32 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, терапия, урология, онкология, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
+          <t>стоматология, детская стоматология, имплантация, протезирование, пародонтология, гигиена, хирургия, ортопедическая стоматология</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Направления деятельности</t>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>5406137478</t>
+          <t>6658006884</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -10316,32 +10831,32 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, лечение бесплодия (ЭКО), общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, лучевая диагностика, терапия, урология, ультразвуковая диагностика, стоматология, онкология, восстановительное лечение, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
+          <t>стоматология</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр 'АВИЦЕННА' - частная клиника мирового уровня в Новосибирске</t>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, ООО</t>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>7204082420</t>
+          <t>6658006884</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -10351,37 +10866,37 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Аллергология и иммунология, Акушерство и гинекология, Гастроэнтерология, Дерматовенерология / дерматология, Кардиология, Неврология, Отоларингология (ЛОР), Офтальмология, Подология, Пульмонология, Ревматология, Рентгенологические исследования, Стоматология, Терапия (общая), Трихология, УЗИ диагностика, Урология, Физиотерапия, Фитотерапия, Эндокринология, Гирудотерапия, Криотерапия, Лабораторная диагностика, Функциональная диагностика</t>
+          <t>стоматология</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, ООО</t>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>7204082420</t>
+          <t>5406513676</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -10396,32 +10911,32 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>аллергология, гинекология</t>
+          <t>Диагностическое отделение, Консультативное отделение, Косметологическое отделение, Педиатрическое отделение, Хирургическое отделение</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности</t>
+          <t>Лечебно-диагностический центр «АвисМед»</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, ООО</t>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>7204082420</t>
+          <t>5406513676</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -10436,32 +10951,32 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>аллергология-иммунология, акушерство-гинекология, гастроэнтерология, дерматовенерология, кардиология, неврология, отоларингология, офтальмология, пульмонология, ревматология, стоматология, терапия, эндокринология</t>
+          <t>дерматология, косметология</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
+          <t>Лечебно-диагностический центр «АвисМед», специалисты: гинеколог, дерматолог, косметолог, невролог, онколог, оториноларинголог, педиатр, стоматолог, терапевт, уролог, флеболог, хирург</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>АВК-МЕД, ООО</t>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>5260156369</t>
+          <t>5406513676</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -10471,37 +10986,37 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>иммунология, терапия, хирургия, кардиология, гастроэнтерология, лабораторная диагностика</t>
+          <t>гинекология, дерматология, косметология, неврология, онкология, оториноларингология, педиатрия, стоматология, терапия, урология, флебология, хирургия</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Специальности врачей: иммунолог, терапевт, хирург; позиции прайса включают Болезнь Крона, Артериальная гипертония, анализы крови и другие медицинские услуги.</t>
+          <t>Записаться на услуги лечебно-диагностического центра «АвисМед»</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>АВК-МЕД, ООО</t>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>5260156369</t>
+          <t>1653000230</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -10516,32 +11031,32 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>иммунология, терапия, хирургия, кардиология</t>
+          <t>эндокринология, детская эндокринология, кардиология, терапия, ультразвуковая диагностика, гастроэнтерология, детская гастроэнтерология, андрология‑урология, детская урология‑андрология, акушер‑гинекология, детская акушер‑гинекология, неврология, детская неврология, остеопатия, детская остеопатия, мануальная терапия, сосудистый хирург‑флебология, онкология, маммология, хирургия (включая ожоговый хирург), нефрология, детская нефрология, психотерапия, детская психотерапия, массаж, нутрициология, офтальмология, детская офтальмология, функциональная диагностика, травматология‑ортопедия, педиатрия, дерматология, детская дерматология, генетические исследования, криодеструкция, биоимпедансометрия, физиотерапия, озонотерапия, склеротерапия, краниосакральная терапия</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Позиции прайса: Болезнь Крона, Артериальная гипертония, Атеросклероз, Профиль №45 "Сердечно-сосудистые заболевания"</t>
+          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>АВК-МЕД, ООО</t>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>5260156369</t>
+          <t>1653000230</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -10556,32 +11071,32 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>иммунология, терапия, хирургия</t>
+          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>https://avk-med.inni.info/produkt/meditsinskiye-uslugi-analizy-meditsinskiye: «ул. Ошарская, д.14-В»</t>
+          <t>Услуги: Эндокринолог, Гастроэнтеролог, Гинеколог, Дерматолог, Кардиолог, Невролог, Онколог, Офтальмолог, Педиатр, Психотерапевт, Терапевт, Уролог, Флеболог, Хирург</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>АВТО-МЕД, ООО</t>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>6324110942</t>
+          <t>1653000230</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -10591,37 +11106,37 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>флебология, хирургия</t>
+          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
+          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>АВТО-МЕД, ООО</t>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>6324110942</t>
+          <t>5406137478</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -10631,37 +11146,37 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>флебология</t>
+          <t>гинекология, кардиология и сердечно‑сосудистая хирургия, неврология и нейрохирургия, травматология и ортопедия, урология, онкология, оториноларингология, офтальмология и микрохирургия глаза, пластическая и реконструктивная хирургия, педиатрия, терапия, стоматология, лечения бесплодия (ЭКО), лабораторная и генетическая диагностика, лучевая диагностика, восстановительное лечение</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
+          <t>TITLE: Медицинский центр "АВИЦЕННА" - частная клиника мирового уровня в Новосибирске; меню сайта содержит разделы «Клиника гинекологическое», «Клиника кардиологии», «Клиника неврологии», «Клиника онкологии» и др., а также ссылки «Лицензии».</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>АВТО-МЕД, ООО</t>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>6324110942</t>
+          <t>5406137478</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -10671,37 +11186,37 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>флебология, хирургия</t>
+          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, терапия, урология, онкология, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб!</t>
+          <t>Направления деятельности</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>5407494063</t>
+          <t>5406137478</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -10716,32 +11231,32 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>пластическая хирургия, косметология, диетология, сомнология, мезотерапия, пилинг, инъекционная косметология, аппаратная косметология, хирургия груди, хирургия тела, хирургия лица, биоимпедансометрия, похудение</t>
+          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, лечение бесплодия (ЭКО), общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, лучевая диагностика, терапия, урология, ультразвуковая диагностика, стоматология, онкология, восстановительное лечение, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
+          <t>Медицинский центр 'АВИЦЕННА' - частная клиника мирового уровня в Новосибирске</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+          <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>5407494063</t>
+          <t>7204082420</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -10751,37 +11266,37 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>косметология, пластическая хирургия</t>
+          <t>Аллергология и иммунология, Акушерство и гинекология, Гастроэнтерология, Дерматовенерология / дерматология, Кардиология, Неврология, Отоларингология (ЛОР), Офтальмология, Подология, Пульмонология, Ревматология, Рентгенологические исследования, Стоматология, Терапия (общая), Трихология, УЗИ диагностика, Урология, Физиотерапия, Фитотерапия, Эндокринология, Гирудотерапия, Криотерапия, Лабораторная диагностика, Функциональная диагностика</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Лицензия №1, Приложение к лицензии №1, Приложение к лицензии №2-1, Приложение к лицензии №2-2, Приложение к лицензии №2-3, Лицензия №2</t>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+          <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>5407494063</t>
+          <t>7204082420</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -10791,37 +11306,37 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>пластическая хирургия, врачебная косметология, диетология, сомнология</t>
+          <t>аллергология, гинекология</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>АГК, ООО</t>
+          <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>2461016768</t>
+          <t>7204082420</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -10831,37 +11346,37 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Акушерство и гинекология, Андрология и урология, Лабораторная диагностика, Физиотерапия, Ультразвуковая диагностика, Хирургия, Сосудистая хирургия, Оперативная гинекология, Проктология, Эндоскопия, Маммология и онкология, Плазмолифтинг, Терапевт</t>
+          <t>аллергология-иммунология, акушерство-гинекология, гастроэнтерология, дерматовенерология, кардиология, неврология, отоларингология, офтальмология, пульмонология, ревматология, стоматология, терапия, эндокринология</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>«Клиника лицензирована и соответствует всем требованиям медицинской безопасности»</t>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>АГК, ООО</t>
+          <t>АВК-МЕД, ООО</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>2461016768</t>
+          <t>5260156369</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -10876,32 +11391,32 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, хирургия, онкология, терапия</t>
+          <t>иммунология, терапия, хирургия, кардиология, гастроэнтерология, лабораторная диагностика</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Услуги центра: Акушерство и гинекология, Андрология и Урология, Хирургия, Маммология и онкология, Терапевт</t>
+          <t>Специальности врачей: иммунолог, терапевт, хирург; позиции прайса включают Болезнь Крона, Артериальная гипертония, анализы крови и другие медицинские услуги.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>АГК, ООО</t>
+          <t>АВК-МЕД, ООО</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>2461016768</t>
+          <t>5260156369</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -10916,32 +11431,32 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>акушерство и гинекология, андрология и урология, лабораторная диагностика, физиотерапия, ультразвуковая диагностика, хирургия, сосудистая хирургия, оперативная гинекология, проктология, эндоскопия, маммология и онкология, терапия</t>
+          <t>иммунология, терапия, хирургия, кардиология</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>ООО 'АГК' - первая частная клиника в Красноярске, занимающаяся вопросами мужского и женского здоровья с 1997г. Клиника лицензирована и соответствует всем требованиям медицинской безопасности.</t>
+          <t>Позиции прайса: Болезнь Крона, Артериальная гипертония, Атеросклероз, Профиль №45 "Сердечно-сосудистые заболевания"</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АВК-МЕД, ООО</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>7813610598</t>
+          <t>5260156369</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -10956,37 +11471,37 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, УЗИ, ЭКГ, Мануальная терапия, Психиатрия детская</t>
+          <t>иммунология, терапия, хирургия</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>https://avk-med.inni.info/produkt/meditsinskiye-uslugi-analizy-meditsinskiye: «ул. Ошарская, д.14-В»</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АВРОРА, ООО</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>7813610598</t>
+          <t>6164209193</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -10994,39 +11509,35 @@
           <t>не определено</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>общая практика, дерматология, стоматология</t>
-        </is>
-      </c>
+      <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>TITLE: Купить автомобиль в Ростове-на-Дону - автосалон Аврора</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АВРОРА, ООО</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>7813610598</t>
+          <t>6164209193</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>yandexgpt</t>
+          <t>llm7</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -11034,39 +11545,35 @@
           <t>не определено</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
-        </is>
-      </c>
+      <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
+          <t>TITLE: Купить автомобиль в Ростове-на-Дону - автосалон Аврора</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АВРОРА, ООО</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>6314040975</t>
+          <t>6164209193</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>yandexgpt</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -11074,34 +11581,30 @@
           <t>не определено</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, Мануальная терапия, Психиатрия детская, УЗИ, ЭКГ</t>
-        </is>
-      </c>
+      <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>Компания занимается продажей автомобилей, что подтверждается заголовками и описанием на сайте.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АВТО-МЕД, ООО</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>6314040975</t>
+          <t>6324110942</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>llm7</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -11111,55 +11614,815 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>общая практика, дерматология, стоматология</t>
+          <t>флебология, хирургия</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>АВТО-МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>6324110942</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>флебология</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>АВТО-МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>6324110942</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>флебология, хирургия</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб!</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>5407494063</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>пластическая хирургия, косметология, диетология, сомнология, мезотерапия, пилинг, инъекционная косметология, аппаратная косметология, хирургия груди, хирургия тела, хирургия лица, биоимпедансометрия, похудение</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>5407494063</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>косметология, пластическая хирургия</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Лицензия №1, Приложение к лицензии №1, Приложение к лицензии №2-1, Приложение к лицензии №2-2, Приложение к лицензии №2-3, Лицензия №2</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>5407494063</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>пластическая хирургия, врачебная косметология, диетология, сомнология</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>АГАТ, ООО</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>6162081830</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>аллергология, иммунология, анестезиология, реаниматология, гастроэнтерология, гинекология, дерматология, косметология, трихология, кардиология, неврология, онкология, оториноларингология, офтальмология, педиатрия, пульмонология, ревматология, терапия, урология, флебология, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение. Специальности врачей: аллерголог, гастроэнтеролог, гинеколог, дерматолог, косметолог, невролог, онколог, педиатр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>АГАТ, ООО</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>6162081830</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>аллергология-иммунология, анестезиология-реаниматология</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>На сайте mc-semya.ru указаны страницы с услугами аллергологии-иммунологии и анестезиологии-реаниматологии, что является явным медицинским признаком.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>АГАТ, ООО</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>6162081830</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>аллергология-иммунология, анестезиология и реаниматология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, оториноларингология, офтальмология, педиатрия, пульмонология, ревматология, терапия, трихология, урология, флебология, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>АГК, ООО</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>2461016768</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Акушерство и гинекология, Андрология и урология, Лабораторная диагностика, Физиотерапия, Ультразвуковая диагностика, Хирургия, Сосудистая хирургия, Оперативная гинекология, Проктология, Эндоскопия, Маммология и онкология, Плазмолифтинг, Терапевт</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>«Клиника лицензирована и соответствует всем требованиям медицинской безопасности»</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>АГК, ООО</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>2461016768</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>гинекология, урология, хирургия, онкология, терапия</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Услуги центра: Акушерство и гинекология, Андрология и Урология, Хирургия, Маммология и онкология, Терапевт</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>АГК, ООО</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>2461016768</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>акушерство и гинекология, андрология и урология, лабораторная диагностика, физиотерапия, ультразвуковая диагностика, хирургия, сосудистая хирургия, оперативная гинекология, проктология, эндоскопия, маммология и онкология, терапия</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>ООО 'АГК' - первая частная клиника в Красноярске, занимающаяся вопросами мужского и женского здоровья с 1997г. Клиника лицензирована и соответствует всем требованиям медицинской безопасности.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>аллергология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, отоларингология, офтальмология, педиатрия, психотерапия, пульмонология, ревматология, стоматология, терапия, трихология, урология, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Многопрофильные клиники «Смитра» в Новосибирске; специальные направления врачей: аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уроло</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>дерматология, косметология, трихология</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>На сайте указаны специальности врачей, в том числе дерматолог, косметолог и трихолог, что является явным медицинским признаком.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>аллергология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, отоларингология, офтальмология, педиатрия, психотерапия, пульмонология, ревматология, стоматология, терапия, трихология, урология, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Лицензия (https://smitra.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, УЗИ, ЭКГ, Мануальная терапия, Психиатрия детская</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>общая практика, дерматология, стоматология</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
         <is>
           <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>6314040975</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, Мануальная терапия, Психиатрия детская, УЗИ, ЭКГ</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>6314040975</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>общая практика, дерматология, стоматология</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>6314040975</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>yandexgpt</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t>медорганизация</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>не определено</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr">
+      <c r="G99" s="2" t="inlineStr">
         <is>
           <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
+      <c r="H99" s="2" t="inlineStr">
         <is>
           <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
         </is>
@@ -12072,7 +13335,7 @@
       <c r="Z8" s="2" t="inlineStr"/>
       <c r="AA8" s="2" t="inlineStr"/>
       <c r="AB8" s="2" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -12250,7 +13513,7 @@
       <c r="Z10" s="2" t="inlineStr"/>
       <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -12718,25 +13981,65 @@
           <t>Красноярск</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr"/>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>vesna24.ru</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 2465176508 найден на сайте</t>
+        </is>
+      </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T15" s="2" t="inlineStr"/>
-      <c r="U15" s="2" t="inlineStr"/>
-      <c r="V15" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W15" s="2" t="inlineStr"/>
-      <c r="X15" s="2" t="inlineStr"/>
-      <c r="Y15" s="2" t="inlineStr"/>
-      <c r="Z15" s="2" t="inlineStr"/>
-      <c r="AA15" s="2" t="inlineStr"/>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>Фототерапия</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>косметолог, онколог, хирург</t>
+        </is>
+      </c>
       <c r="AB15" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -13206,25 +14509,61 @@
           <t>Тюмень</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="inlineStr"/>
-      <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>venum-center.ru</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Тюмень (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T20" s="2" t="inlineStr"/>
-      <c r="U20" s="2" t="inlineStr"/>
-      <c r="V20" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>лицензия (мед-контекст): «Лицензия № Л041-01107-72/00361525» (https://venum-center.ru)</t>
+        </is>
+      </c>
       <c r="W20" s="2" t="inlineStr"/>
-      <c r="X20" s="2" t="inlineStr"/>
-      <c r="Y20" s="2" t="inlineStr"/>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z20" s="2" t="inlineStr"/>
-      <c r="AA20" s="2" t="inlineStr"/>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>флеболог, хирург</t>
+        </is>
+      </c>
       <c r="AB20" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
@@ -13390,25 +14729,57 @@
           <t>Уфа</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr"/>
-      <c r="P22" s="2" t="inlineStr"/>
-      <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>grandavenue.ru</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Уфа (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T22" s="2" t="inlineStr"/>
-      <c r="U22" s="2" t="inlineStr"/>
-      <c r="V22" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>медицинских признаков на сайте нет: ни лицензии, ни врачей, ни приёмов (https://grandavenue.ru)</t>
+        </is>
+      </c>
       <c r="W22" s="2" t="inlineStr"/>
-      <c r="X22" s="2" t="inlineStr"/>
-      <c r="Y22" s="2" t="inlineStr"/>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z22" s="2" t="inlineStr"/>
       <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="23">
@@ -13474,7 +14845,7 @@
       <c r="Z23" s="2" t="inlineStr"/>
       <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -14156,25 +15527,57 @@
           <t>Ростов-на-Дону</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr"/>
-      <c r="P30" s="2" t="inlineStr"/>
-      <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>avr-rostov.ru</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Ростов-на-Дону (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T30" s="2" t="inlineStr"/>
-      <c r="U30" s="2" t="inlineStr"/>
-      <c r="V30" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W30" s="2" t="inlineStr"/>
-      <c r="X30" s="2" t="inlineStr"/>
-      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z30" s="2" t="inlineStr"/>
       <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
@@ -14514,13 +15917,29 @@
           <t>Нижний Новгород</t>
         </is>
       </c>
-      <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
-      <c r="R34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>avtotranskontejner.clients.site</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>адрес места деятельности из лицензии РЗН («кузбасская, 1») найден на сайте</t>
+        </is>
+      </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="T34" s="2" t="inlineStr"/>
@@ -14532,7 +15951,7 @@
       <c r="Z34" s="2" t="inlineStr"/>
       <c r="AA34" s="2" t="inlineStr"/>
       <c r="AB34" s="2" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35">
@@ -14598,7 +16017,7 @@
       <c r="Z35" s="2" t="inlineStr"/>
       <c r="AA35" s="2" t="inlineStr"/>
       <c r="AB35" s="2" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36">
@@ -14646,25 +16065,61 @@
           <t>Ростов-на-Дону</t>
         </is>
       </c>
-      <c r="O36" s="2" t="inlineStr"/>
-      <c r="P36" s="2" t="inlineStr"/>
-      <c r="Q36" s="2" t="inlineStr"/>
-      <c r="R36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>mc-semya.ru</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 6162081830 найден на сайте</t>
+        </is>
+      </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T36" s="2" t="inlineStr"/>
-      <c r="U36" s="2" t="inlineStr"/>
-      <c r="V36" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W36" s="2" t="inlineStr"/>
-      <c r="X36" s="2" t="inlineStr"/>
-      <c r="Y36" s="2" t="inlineStr"/>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="Y36" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z36" s="2" t="inlineStr"/>
-      <c r="AA36" s="2" t="inlineStr"/>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, оториноларинголог, офтальмолог, педиатр, пульмонолог, ревматолог, терапевт, трихолог, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="AB36" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37">
@@ -14730,7 +16185,7 @@
       <c r="Z37" s="2" t="inlineStr"/>
       <c r="AA37" s="2" t="inlineStr"/>
       <c r="AB37" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38">
@@ -14902,29 +16357,65 @@
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="O39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>кандидаты выгрузки не подтвердились (гибко)</t>
-        </is>
-      </c>
-      <c r="Q39" s="2" t="inlineStr"/>
-      <c r="R39" s="2" t="inlineStr"/>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>адрес места деятельности из лицензии РЗН («геодезическая, 2/1») найден на сайте</t>
+        </is>
+      </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T39" s="2" t="inlineStr"/>
-      <c r="U39" s="2" t="inlineStr"/>
-      <c r="V39" s="2" t="inlineStr"/>
-      <c r="W39" s="2" t="inlineStr"/>
-      <c r="X39" s="2" t="inlineStr"/>
-      <c r="Y39" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>«…/news/cherno-belaya-vecherinka-kommersant-sibir-shakhmaty-klassika-i-zabota-o-zdorove-ot-kliniki-smitra/)  [![Image 57: Сеть клиник «Смитра» признана лучшей в здравоохранении на городском конкурсе](https://smitra.ru/upload/webp/upload/iblock/f1d/79x9y5vtvwfiecyksen2q2yv5k2aiqpa.webp)](https://smitra.ru/news/set-klinik-smitra-priznana-luchshey-v-zdravookhranenii-na-goro…» (https://smitra.ru)</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>/news/cherno-belaya-vecherinka-kommersant-sibir-shakhmaty-klassika-i-zabota-o-zdorove-ot-kliniki-smitra/)  [![Image 57: Сеть клиник «Смитра» признана лучшей в здравоохранении на городском конкурсе](https://smitra.ru/upload/webp/upload/iblock/f1d/79x9y5vtvwfiecyksen2q2yv5k2aiqpa.webp)](https://smitra</t>
+        </is>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z39" s="2" t="inlineStr"/>
-      <c r="AA39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уролог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="AB39" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40">

</xml_diff>